<commit_message>
Patlıcanlı Sarma ürününü Tuzlu Kurabiye sayfasına ekle
</commit_message>
<xml_diff>
--- a/rapor-duzeni.xlsx
+++ b/rapor-duzeni.xlsx
@@ -500,7 +500,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H220"/>
+  <dimension ref="A1:H221"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4836,34 +4836,32 @@
       </c>
     </row>
     <row r="144">
-      <c r="A144" s="11" t="inlineStr">
+      <c r="A144" t="inlineStr">
         <is>
           <t>Tuzlu Kurabiye</t>
         </is>
       </c>
-      <c r="B144" s="11" t="inlineStr">
+      <c r="B144" t="inlineStr">
         <is>
           <t>Börekli Taş &amp; Poğaça Grubu</t>
         </is>
       </c>
-      <c r="C144" s="11" t="inlineStr">
-        <is>
-          <t>Zeytinli</t>
-        </is>
-      </c>
-      <c r="D144" s="4" t="n">
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>Patlıcanlı Sarma</t>
+        </is>
+      </c>
+      <c r="D144" t="n">
         <v>3</v>
       </c>
-      <c r="E144" s="5" t="inlineStr">
+      <c r="E144" t="inlineStr">
         <is>
           <t>tp</t>
         </is>
       </c>
-      <c r="F144" s="5" t="n"/>
-      <c r="G144" s="9" t="n"/>
-      <c r="H144" s="11" t="inlineStr">
-        <is>
-          <t>Zeytinli</t>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>Patlıcanlı Sarma</t>
         </is>
       </c>
     </row>
@@ -4880,7 +4878,7 @@
       </c>
       <c r="C145" s="11" t="inlineStr">
         <is>
-          <t>Patatesli</t>
+          <t>Zeytinli</t>
         </is>
       </c>
       <c r="D145" s="4" t="n">
@@ -4895,7 +4893,7 @@
       <c r="G145" s="9" t="n"/>
       <c r="H145" s="11" t="inlineStr">
         <is>
-          <t>Patatesli</t>
+          <t>Zeytinli</t>
         </is>
       </c>
     </row>
@@ -4912,7 +4910,7 @@
       </c>
       <c r="C146" s="11" t="inlineStr">
         <is>
-          <t>Kornet Dereotlu</t>
+          <t>Patatesli</t>
         </is>
       </c>
       <c r="D146" s="4" t="n">
@@ -4920,14 +4918,14 @@
       </c>
       <c r="E146" s="5" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>tp</t>
         </is>
       </c>
       <c r="F146" s="5" t="n"/>
       <c r="G146" s="9" t="n"/>
       <c r="H146" s="11" t="inlineStr">
         <is>
-          <t>Kornet Dereotlu</t>
+          <t>Patatesli</t>
         </is>
       </c>
     </row>
@@ -4944,7 +4942,7 @@
       </c>
       <c r="C147" s="11" t="inlineStr">
         <is>
-          <t>Dereotlu Sufle</t>
+          <t>Kornet Dereotlu</t>
         </is>
       </c>
       <c r="D147" s="4" t="n">
@@ -4959,7 +4957,7 @@
       <c r="G147" s="9" t="n"/>
       <c r="H147" s="11" t="inlineStr">
         <is>
-          <t>Dereotlu Sufle</t>
+          <t>Kornet Dereotlu</t>
         </is>
       </c>
     </row>
@@ -4976,7 +4974,7 @@
       </c>
       <c r="C148" s="11" t="inlineStr">
         <is>
-          <t>Sebzeli</t>
+          <t>Dereotlu Sufle</t>
         </is>
       </c>
       <c r="D148" s="4" t="n">
@@ -4984,14 +4982,14 @@
       </c>
       <c r="E148" s="5" t="inlineStr">
         <is>
-          <t>tp</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="F148" s="5" t="n"/>
       <c r="G148" s="9" t="n"/>
       <c r="H148" s="11" t="inlineStr">
         <is>
-          <t>Sebzeli</t>
+          <t>Dereotlu Sufle</t>
         </is>
       </c>
     </row>
@@ -5008,7 +5006,7 @@
       </c>
       <c r="C149" s="11" t="inlineStr">
         <is>
-          <t>Patlıcanlı</t>
+          <t>Sebzeli</t>
         </is>
       </c>
       <c r="D149" s="4" t="n">
@@ -5023,7 +5021,7 @@
       <c r="G149" s="9" t="n"/>
       <c r="H149" s="11" t="inlineStr">
         <is>
-          <t>Patlıcanlı</t>
+          <t>Sebzeli</t>
         </is>
       </c>
     </row>
@@ -5040,7 +5038,7 @@
       </c>
       <c r="C150" s="11" t="inlineStr">
         <is>
-          <t>Mini Pizza</t>
+          <t>Patlıcanlı</t>
         </is>
       </c>
       <c r="D150" s="4" t="n">
@@ -5055,7 +5053,7 @@
       <c r="G150" s="9" t="n"/>
       <c r="H150" s="11" t="inlineStr">
         <is>
-          <t>Mini Pizza</t>
+          <t>Patlıcanlı</t>
         </is>
       </c>
     </row>
@@ -5072,7 +5070,7 @@
       </c>
       <c r="C151" s="11" t="inlineStr">
         <is>
-          <t>Minik Simit</t>
+          <t>Mini Pizza</t>
         </is>
       </c>
       <c r="D151" s="4" t="n">
@@ -5087,7 +5085,7 @@
       <c r="G151" s="9" t="n"/>
       <c r="H151" s="11" t="inlineStr">
         <is>
-          <t>Minik Simit</t>
+          <t>Mini Pizza</t>
         </is>
       </c>
     </row>
@@ -5104,7 +5102,7 @@
       </c>
       <c r="C152" s="11" t="inlineStr">
         <is>
-          <t>Düz Örgü</t>
+          <t>Minik Simit</t>
         </is>
       </c>
       <c r="D152" s="4" t="n">
@@ -5119,7 +5117,7 @@
       <c r="G152" s="9" t="n"/>
       <c r="H152" s="11" t="inlineStr">
         <is>
-          <t>Düz Örgü</t>
+          <t>Minik Simit</t>
         </is>
       </c>
     </row>
@@ -5136,7 +5134,7 @@
       </c>
       <c r="C153" s="11" t="inlineStr">
         <is>
-          <t>Yuvarlak Örgü</t>
+          <t>Düz Örgü</t>
         </is>
       </c>
       <c r="D153" s="4" t="n">
@@ -5151,7 +5149,7 @@
       <c r="G153" s="9" t="n"/>
       <c r="H153" s="11" t="inlineStr">
         <is>
-          <t>Yuvarlak Örgü</t>
+          <t>Düz Örgü</t>
         </is>
       </c>
     </row>
@@ -5168,7 +5166,7 @@
       </c>
       <c r="C154" s="11" t="inlineStr">
         <is>
-          <t>Burgu Susamlı Haşhaşlı</t>
+          <t>Yuvarlak Örgü</t>
         </is>
       </c>
       <c r="D154" s="4" t="n">
@@ -5183,67 +5181,67 @@
       <c r="G154" s="9" t="n"/>
       <c r="H154" s="11" t="inlineStr">
         <is>
+          <t>Yuvarlak Örgü</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="11" t="inlineStr">
+        <is>
+          <t>Tuzlu Kurabiye</t>
+        </is>
+      </c>
+      <c r="B155" s="11" t="inlineStr">
+        <is>
+          <t>Börekli Taş &amp; Poğaça Grubu</t>
+        </is>
+      </c>
+      <c r="C155" s="11" t="inlineStr">
+        <is>
           <t>Burgu Susamlı Haşhaşlı</t>
         </is>
       </c>
-    </row>
-    <row r="155">
-      <c r="A155" s="2" t="inlineStr">
-        <is>
-          <t>Tuzlu Kurabiye</t>
-        </is>
-      </c>
-      <c r="B155" s="2" t="inlineStr">
-        <is>
-          <t>Diyet Kurabiyeler</t>
-        </is>
-      </c>
-      <c r="C155" s="11" t="inlineStr">
-        <is>
-          <t>Burgu Tahıllı</t>
-        </is>
-      </c>
       <c r="D155" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E155" s="5" t="n"/>
+        <v>14</v>
+      </c>
+      <c r="E155" s="5" t="inlineStr">
+        <is>
+          <t>tp</t>
+        </is>
+      </c>
       <c r="F155" s="5" t="n"/>
       <c r="G155" s="9" t="n"/>
       <c r="H155" s="11" t="inlineStr">
         <is>
+          <t>Burgu Susamlı Haşhaşlı</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="2" t="inlineStr">
+        <is>
+          <t>Tuzlu Kurabiye</t>
+        </is>
+      </c>
+      <c r="B156" s="2" t="inlineStr">
+        <is>
+          <t>Diyet Kurabiyeler</t>
+        </is>
+      </c>
+      <c r="C156" s="11" t="inlineStr">
+        <is>
           <t>Burgu Tahıllı</t>
         </is>
       </c>
-    </row>
-    <row r="156">
-      <c r="A156" s="11" t="inlineStr">
-        <is>
-          <t>Tuzlu Kurabiye</t>
-        </is>
-      </c>
-      <c r="B156" s="11" t="inlineStr">
-        <is>
-          <t>Diyet Kurabiyeler</t>
-        </is>
-      </c>
-      <c r="C156" s="11" t="inlineStr">
-        <is>
-          <t>Ayçekirdekli Galeta</t>
-        </is>
-      </c>
       <c r="D156" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="E156" s="5" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="E156" s="5" t="n"/>
       <c r="F156" s="5" t="n"/>
       <c r="G156" s="9" t="n"/>
       <c r="H156" s="11" t="inlineStr">
         <is>
-          <t>Ayçekirdekli Galeta</t>
+          <t>Burgu Tahıllı</t>
         </is>
       </c>
     </row>
@@ -5260,22 +5258,22 @@
       </c>
       <c r="C157" s="11" t="inlineStr">
         <is>
-          <t>Parmesan Galeta</t>
+          <t>Ayçekirdekli Galeta</t>
         </is>
       </c>
       <c r="D157" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E157" s="5" t="inlineStr">
         <is>
-          <t>tp</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="F157" s="5" t="n"/>
       <c r="G157" s="9" t="n"/>
       <c r="H157" s="11" t="inlineStr">
         <is>
-          <t>Parmesan Galeta</t>
+          <t>Ayçekirdekli Galeta</t>
         </is>
       </c>
     </row>
@@ -5292,11 +5290,11 @@
       </c>
       <c r="C158" s="11" t="inlineStr">
         <is>
-          <t>İtalyan Galeta</t>
+          <t>Parmesan Galeta</t>
         </is>
       </c>
       <c r="D158" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E158" s="5" t="inlineStr">
         <is>
@@ -5307,7 +5305,7 @@
       <c r="G158" s="9" t="n"/>
       <c r="H158" s="11" t="inlineStr">
         <is>
-          <t>İtalyan Galeta</t>
+          <t>Parmesan Galeta</t>
         </is>
       </c>
     </row>
@@ -5324,11 +5322,11 @@
       </c>
       <c r="C159" s="11" t="inlineStr">
         <is>
-          <t>Biberiyeli Zeytinli Galeta</t>
+          <t>İtalyan Galeta</t>
         </is>
       </c>
       <c r="D159" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E159" s="5" t="inlineStr">
         <is>
@@ -5339,7 +5337,7 @@
       <c r="G159" s="9" t="n"/>
       <c r="H159" s="11" t="inlineStr">
         <is>
-          <t>Biberiyeli Zeytinli Galeta</t>
+          <t>İtalyan Galeta</t>
         </is>
       </c>
     </row>
@@ -5356,11 +5354,11 @@
       </c>
       <c r="C160" s="11" t="inlineStr">
         <is>
-          <t>Çekirdekli Kokteyl</t>
+          <t>Biberiyeli Zeytinli Galeta</t>
         </is>
       </c>
       <c r="D160" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E160" s="5" t="inlineStr">
         <is>
@@ -5371,7 +5369,7 @@
       <c r="G160" s="9" t="n"/>
       <c r="H160" s="11" t="inlineStr">
         <is>
-          <t>Çekirdekli Kokteyl</t>
+          <t>Biberiyeli Zeytinli Galeta</t>
         </is>
       </c>
     </row>
@@ -5388,11 +5386,11 @@
       </c>
       <c r="C161" s="11" t="inlineStr">
         <is>
-          <t>Üzümlü Kepekli</t>
+          <t>Çekirdekli Kokteyl</t>
         </is>
       </c>
       <c r="D161" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E161" s="5" t="inlineStr">
         <is>
@@ -5403,7 +5401,7 @@
       <c r="G161" s="9" t="n"/>
       <c r="H161" s="11" t="inlineStr">
         <is>
-          <t>Üzümlü Kepekli</t>
+          <t>Çekirdekli Kokteyl</t>
         </is>
       </c>
     </row>
@@ -5420,11 +5418,11 @@
       </c>
       <c r="C162" s="11" t="inlineStr">
         <is>
-          <t>Üzümlü Cevizli Kepekli</t>
+          <t>Üzümlü Kepekli</t>
         </is>
       </c>
       <c r="D162" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E162" s="5" t="inlineStr">
         <is>
@@ -5435,7 +5433,7 @@
       <c r="G162" s="9" t="n"/>
       <c r="H162" s="11" t="inlineStr">
         <is>
-          <t>Üzümlü Cevizli Kepekli</t>
+          <t>Üzümlü Kepekli</t>
         </is>
       </c>
     </row>
@@ -5452,18 +5450,22 @@
       </c>
       <c r="C163" s="11" t="inlineStr">
         <is>
-          <t>Kuru Üzümlü Yassı Tahıllı</t>
+          <t>Üzümlü Cevizli Kepekli</t>
         </is>
       </c>
       <c r="D163" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="E163" s="5" t="n"/>
+        <v>8</v>
+      </c>
+      <c r="E163" s="5" t="inlineStr">
+        <is>
+          <t>tp</t>
+        </is>
+      </c>
       <c r="F163" s="5" t="n"/>
       <c r="G163" s="9" t="n"/>
       <c r="H163" s="11" t="inlineStr">
         <is>
-          <t>Kuru Üzümlü Yassı Tahıllı</t>
+          <t>Üzümlü Cevizli Kepekli</t>
         </is>
       </c>
     </row>
@@ -5480,22 +5482,18 @@
       </c>
       <c r="C164" s="11" t="inlineStr">
         <is>
-          <t>Granola Bar Tepsi</t>
+          <t>Kuru Üzümlü Yassı Tahıllı</t>
         </is>
       </c>
       <c r="D164" s="4" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E164" s="5" t="n"/>
       <c r="F164" s="5" t="n"/>
-      <c r="G164" s="9" t="inlineStr">
-        <is>
-          <t>Bar</t>
-        </is>
-      </c>
+      <c r="G164" s="9" t="n"/>
       <c r="H164" s="11" t="inlineStr">
         <is>
-          <t>Granola Bar Tepsi</t>
+          <t>Kuru Üzümlü Yassı Tahıllı</t>
         </is>
       </c>
     </row>
@@ -5512,18 +5510,22 @@
       </c>
       <c r="C165" s="11" t="inlineStr">
         <is>
-          <t>Tahinli Susamlı</t>
+          <t>Granola Bar Tepsi</t>
         </is>
       </c>
       <c r="D165" s="4" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E165" s="5" t="n"/>
       <c r="F165" s="5" t="n"/>
-      <c r="G165" s="9" t="n"/>
+      <c r="G165" s="9" t="inlineStr">
+        <is>
+          <t>Bar</t>
+        </is>
+      </c>
       <c r="H165" s="11" t="inlineStr">
         <is>
-          <t>Tahinli Susamlı</t>
+          <t>Granola Bar Tepsi</t>
         </is>
       </c>
     </row>
@@ -5540,18 +5542,18 @@
       </c>
       <c r="C166" s="11" t="inlineStr">
         <is>
-          <t>Granola Dökme</t>
+          <t>Tahinli Susamlı</t>
         </is>
       </c>
       <c r="D166" s="4" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E166" s="5" t="n"/>
       <c r="F166" s="5" t="n"/>
       <c r="G166" s="9" t="n"/>
       <c r="H166" s="11" t="inlineStr">
         <is>
-          <t>Granola Dökme</t>
+          <t>Tahinli Susamlı</t>
         </is>
       </c>
     </row>
@@ -5568,74 +5570,74 @@
       </c>
       <c r="C167" s="11" t="inlineStr">
         <is>
-          <t>Kalp Denge Tahıllı</t>
+          <t>Granola Dökme</t>
         </is>
       </c>
       <c r="D167" s="4" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E167" s="5" t="n"/>
       <c r="F167" s="5" t="n"/>
       <c r="G167" s="9" t="n"/>
       <c r="H167" s="11" t="inlineStr">
         <is>
+          <t>Granola Dökme</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="11" t="inlineStr">
+        <is>
+          <t>Tuzlu Kurabiye</t>
+        </is>
+      </c>
+      <c r="B168" s="11" t="inlineStr">
+        <is>
+          <t>Diyet Kurabiyeler</t>
+        </is>
+      </c>
+      <c r="C168" s="11" t="inlineStr">
+        <is>
           <t>Kalp Denge Tahıllı</t>
         </is>
       </c>
-    </row>
-    <row r="168">
-      <c r="A168" s="2" t="inlineStr">
-        <is>
-          <t>Tuzlu Kurabiye</t>
-        </is>
-      </c>
-      <c r="B168" s="2" t="inlineStr">
-        <is>
-          <t>Adet Ürünler</t>
-        </is>
-      </c>
-      <c r="C168" s="11" t="inlineStr">
-        <is>
-          <t>Paskalya</t>
-        </is>
-      </c>
       <c r="D168" s="4" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="E168" s="5" t="n"/>
       <c r="F168" s="5" t="n"/>
       <c r="G168" s="9" t="n"/>
       <c r="H168" s="11" t="inlineStr">
         <is>
+          <t>Kalp Denge Tahıllı</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="2" t="inlineStr">
+        <is>
+          <t>Tuzlu Kurabiye</t>
+        </is>
+      </c>
+      <c r="B169" s="2" t="inlineStr">
+        <is>
+          <t>Adet Ürünler</t>
+        </is>
+      </c>
+      <c r="C169" s="11" t="inlineStr">
+        <is>
           <t>Paskalya</t>
         </is>
       </c>
-    </row>
-    <row r="169">
-      <c r="A169" s="11" t="inlineStr">
-        <is>
-          <t>Tuzlu Kurabiye</t>
-        </is>
-      </c>
-      <c r="B169" s="11" t="inlineStr">
-        <is>
-          <t>Adet Ürünler</t>
-        </is>
-      </c>
-      <c r="C169" s="11" t="inlineStr">
-        <is>
-          <t>Paskalya Çikolatalı</t>
-        </is>
-      </c>
       <c r="D169" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E169" s="5" t="n"/>
       <c r="F169" s="5" t="n"/>
       <c r="G169" s="9" t="n"/>
       <c r="H169" s="11" t="inlineStr">
         <is>
-          <t>Paskalya Çikolatalı</t>
+          <t>Paskalya</t>
         </is>
       </c>
     </row>
@@ -5652,18 +5654,18 @@
       </c>
       <c r="C170" s="11" t="inlineStr">
         <is>
-          <t>Tahinli Çörek</t>
+          <t>Paskalya Çikolatalı</t>
         </is>
       </c>
       <c r="D170" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E170" s="5" t="n"/>
       <c r="F170" s="5" t="n"/>
       <c r="G170" s="9" t="n"/>
       <c r="H170" s="11" t="inlineStr">
         <is>
-          <t>Tahinli Çörek</t>
+          <t>Paskalya Çikolatalı</t>
         </is>
       </c>
     </row>
@@ -5680,22 +5682,18 @@
       </c>
       <c r="C171" s="11" t="inlineStr">
         <is>
-          <t>Beze Büyük</t>
+          <t>Tahinli Çörek</t>
         </is>
       </c>
       <c r="D171" s="4" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E171" s="5" t="n"/>
       <c r="F171" s="5" t="n"/>
-      <c r="G171" s="9" t="inlineStr">
-        <is>
-          <t>Beze</t>
-        </is>
-      </c>
+      <c r="G171" s="9" t="n"/>
       <c r="H171" s="11" t="inlineStr">
         <is>
-          <t>Beze Büyük</t>
+          <t>Tahinli Çörek</t>
         </is>
       </c>
     </row>
@@ -5712,11 +5710,11 @@
       </c>
       <c r="C172" s="11" t="inlineStr">
         <is>
-          <t>Beze Beyaz Minik</t>
+          <t>Beze Büyük</t>
         </is>
       </c>
       <c r="D172" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E172" s="5" t="n"/>
       <c r="F172" s="5" t="n"/>
@@ -5727,7 +5725,7 @@
       </c>
       <c r="H172" s="11" t="inlineStr">
         <is>
-          <t>Beze Beyaz Minik</t>
+          <t>Beze Büyük</t>
         </is>
       </c>
     </row>
@@ -5744,11 +5742,11 @@
       </c>
       <c r="C173" s="11" t="inlineStr">
         <is>
-          <t>Beze Renkli Minik</t>
+          <t>Beze Beyaz Minik</t>
         </is>
       </c>
       <c r="D173" s="4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E173" s="5" t="n"/>
       <c r="F173" s="5" t="n"/>
@@ -5759,7 +5757,7 @@
       </c>
       <c r="H173" s="11" t="inlineStr">
         <is>
-          <t>Beze Renkli Minik</t>
+          <t>Beze Beyaz Minik</t>
         </is>
       </c>
     </row>
@@ -5776,18 +5774,22 @@
       </c>
       <c r="C174" s="11" t="inlineStr">
         <is>
-          <t>Acıbadem</t>
+          <t>Beze Renkli Minik</t>
         </is>
       </c>
       <c r="D174" s="4" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="E174" s="5" t="n"/>
       <c r="F174" s="5" t="n"/>
-      <c r="G174" s="9" t="n"/>
+      <c r="G174" s="9" t="inlineStr">
+        <is>
+          <t>Beze</t>
+        </is>
+      </c>
       <c r="H174" s="11" t="inlineStr">
         <is>
-          <t>Acıbadem</t>
+          <t>Beze Renkli Minik</t>
         </is>
       </c>
     </row>
@@ -5804,18 +5806,18 @@
       </c>
       <c r="C175" s="11" t="inlineStr">
         <is>
-          <t>Acıbadem Minik</t>
+          <t>Acıbadem</t>
         </is>
       </c>
       <c r="D175" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E175" s="5" t="n"/>
       <c r="F175" s="5" t="n"/>
       <c r="G175" s="9" t="n"/>
       <c r="H175" s="11" t="inlineStr">
         <is>
-          <t>Acıbadem Minik</t>
+          <t>Acıbadem</t>
         </is>
       </c>
     </row>
@@ -5832,75 +5834,67 @@
       </c>
       <c r="C176" s="11" t="inlineStr">
         <is>
-          <t>Ayçöreği</t>
+          <t>Acıbadem Minik</t>
         </is>
       </c>
       <c r="D176" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E176" s="5" t="n"/>
       <c r="F176" s="5" t="n"/>
       <c r="G176" s="9" t="n"/>
       <c r="H176" s="11" t="inlineStr">
         <is>
+          <t>Acıbadem Minik</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="11" t="inlineStr">
+        <is>
+          <t>Tuzlu Kurabiye</t>
+        </is>
+      </c>
+      <c r="B177" s="11" t="inlineStr">
+        <is>
+          <t>Adet Ürünler</t>
+        </is>
+      </c>
+      <c r="C177" s="11" t="inlineStr">
+        <is>
           <t>Ayçöreği</t>
         </is>
       </c>
-    </row>
-    <row r="177">
-      <c r="A177" s="2" t="inlineStr">
+      <c r="D177" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="E177" s="5" t="n"/>
+      <c r="F177" s="5" t="n"/>
+      <c r="G177" s="9" t="n"/>
+      <c r="H177" s="11" t="inlineStr">
+        <is>
+          <t>Ayçöreği</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="2" t="inlineStr">
         <is>
           <t>Tuzlu Kurabiye</t>
         </is>
       </c>
-      <c r="B177" s="2" t="inlineStr">
+      <c r="B178" s="2" t="inlineStr">
         <is>
           <t>Galeta / Kıtır / Cips / Diğer Tuzlu</t>
         </is>
       </c>
-      <c r="C177" s="11" t="inlineStr">
+      <c r="C178" s="11" t="inlineStr">
         <is>
           <t>Batonsale Sade</t>
         </is>
       </c>
-      <c r="D177" s="4" t="n">
+      <c r="D178" s="4" t="n">
         <v>1</v>
-      </c>
-      <c r="E177" s="5" t="inlineStr">
-        <is>
-          <t>tp</t>
-        </is>
-      </c>
-      <c r="F177" s="5" t="n"/>
-      <c r="G177" s="9" t="inlineStr">
-        <is>
-          <t>Batonsale</t>
-        </is>
-      </c>
-      <c r="H177" s="11" t="inlineStr">
-        <is>
-          <t>Batonsale Sade</t>
-        </is>
-      </c>
-    </row>
-    <row r="178">
-      <c r="A178" s="11" t="inlineStr">
-        <is>
-          <t>Tuzlu Kurabiye</t>
-        </is>
-      </c>
-      <c r="B178" s="11" t="inlineStr">
-        <is>
-          <t>Galeta / Kıtır / Cips / Diğer Tuzlu</t>
-        </is>
-      </c>
-      <c r="C178" s="11" t="inlineStr">
-        <is>
-          <t>Batonsale Çörekotlu</t>
-        </is>
-      </c>
-      <c r="D178" s="4" t="n">
-        <v>2</v>
       </c>
       <c r="E178" s="5" t="inlineStr">
         <is>
@@ -5915,7 +5909,7 @@
       </c>
       <c r="H178" s="11" t="inlineStr">
         <is>
-          <t>Batonsale Çörekotlu</t>
+          <t>Batonsale Sade</t>
         </is>
       </c>
     </row>
@@ -5932,11 +5926,11 @@
       </c>
       <c r="C179" s="11" t="inlineStr">
         <is>
-          <t>Batonsale Kaşarlı</t>
+          <t>Batonsale Çörekotlu</t>
         </is>
       </c>
       <c r="D179" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E179" s="5" t="inlineStr">
         <is>
@@ -5951,7 +5945,7 @@
       </c>
       <c r="H179" s="11" t="inlineStr">
         <is>
-          <t>Batonsale Kaşarlı</t>
+          <t>Batonsale Çörekotlu</t>
         </is>
       </c>
     </row>
@@ -5968,11 +5962,11 @@
       </c>
       <c r="C180" s="11" t="inlineStr">
         <is>
-          <t>Kırık Kırak Susamlı</t>
+          <t>Batonsale Kaşarlı</t>
         </is>
       </c>
       <c r="D180" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E180" s="5" t="inlineStr">
         <is>
@@ -5980,10 +5974,14 @@
         </is>
       </c>
       <c r="F180" s="5" t="n"/>
-      <c r="G180" s="9" t="n"/>
+      <c r="G180" s="9" t="inlineStr">
+        <is>
+          <t>Batonsale</t>
+        </is>
+      </c>
       <c r="H180" s="11" t="inlineStr">
         <is>
-          <t>Kırık Kırak Susamlı</t>
+          <t>Batonsale Kaşarlı</t>
         </is>
       </c>
     </row>
@@ -6000,11 +5998,11 @@
       </c>
       <c r="C181" s="11" t="inlineStr">
         <is>
-          <t>Galet Kaşarlı</t>
+          <t>Kırık Kırak Susamlı</t>
         </is>
       </c>
       <c r="D181" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E181" s="5" t="inlineStr">
         <is>
@@ -6012,14 +6010,10 @@
         </is>
       </c>
       <c r="F181" s="5" t="n"/>
-      <c r="G181" s="9" t="inlineStr">
-        <is>
-          <t>Galet</t>
-        </is>
-      </c>
+      <c r="G181" s="9" t="n"/>
       <c r="H181" s="11" t="inlineStr">
         <is>
-          <t>Galet Kaşarlı</t>
+          <t>Kırık Kırak Susamlı</t>
         </is>
       </c>
     </row>
@@ -6036,11 +6030,11 @@
       </c>
       <c r="C182" s="11" t="inlineStr">
         <is>
-          <t>Galet Çörekotlu</t>
+          <t>Galet Kaşarlı</t>
         </is>
       </c>
       <c r="D182" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E182" s="5" t="inlineStr">
         <is>
@@ -6055,7 +6049,7 @@
       </c>
       <c r="H182" s="11" t="inlineStr">
         <is>
-          <t>Galet Çörekotlu</t>
+          <t>Galet Kaşarlı</t>
         </is>
       </c>
     </row>
@@ -6072,11 +6066,11 @@
       </c>
       <c r="C183" s="11" t="inlineStr">
         <is>
-          <t>Galet Susamlı</t>
+          <t>Galet Çörekotlu</t>
         </is>
       </c>
       <c r="D183" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E183" s="5" t="inlineStr">
         <is>
@@ -6091,7 +6085,7 @@
       </c>
       <c r="H183" s="11" t="inlineStr">
         <is>
-          <t>Galet Susamlı</t>
+          <t>Galet Çörekotlu</t>
         </is>
       </c>
     </row>
@@ -6108,11 +6102,11 @@
       </c>
       <c r="C184" s="11" t="inlineStr">
         <is>
-          <t>Baharatlı Kıtır</t>
+          <t>Galet Susamlı</t>
         </is>
       </c>
       <c r="D184" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E184" s="5" t="inlineStr">
         <is>
@@ -6122,12 +6116,12 @@
       <c r="F184" s="5" t="n"/>
       <c r="G184" s="9" t="inlineStr">
         <is>
-          <t>Kıtır</t>
+          <t>Galet</t>
         </is>
       </c>
       <c r="H184" s="11" t="inlineStr">
         <is>
-          <t>Baharatlı Kıtır</t>
+          <t>Galet Susamlı</t>
         </is>
       </c>
     </row>
@@ -6144,11 +6138,11 @@
       </c>
       <c r="C185" s="11" t="inlineStr">
         <is>
-          <t>Kaşarlı Kıtır</t>
+          <t>Baharatlı Kıtır</t>
         </is>
       </c>
       <c r="D185" s="4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E185" s="5" t="inlineStr">
         <is>
@@ -6163,7 +6157,7 @@
       </c>
       <c r="H185" s="11" t="inlineStr">
         <is>
-          <t>Kaşarlı Kıtır</t>
+          <t>Baharatlı Kıtır</t>
         </is>
       </c>
     </row>
@@ -6180,11 +6174,11 @@
       </c>
       <c r="C186" s="11" t="inlineStr">
         <is>
-          <t>Zencefilli Kıtır</t>
+          <t>Kaşarlı Kıtır</t>
         </is>
       </c>
       <c r="D186" s="4" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E186" s="5" t="inlineStr">
         <is>
@@ -6199,7 +6193,7 @@
       </c>
       <c r="H186" s="11" t="inlineStr">
         <is>
-          <t>Zencefilli Kıtır</t>
+          <t>Kaşarlı Kıtır</t>
         </is>
       </c>
     </row>
@@ -6216,11 +6210,11 @@
       </c>
       <c r="C187" s="11" t="inlineStr">
         <is>
-          <t>Acılı Kıtır</t>
+          <t>Zencefilli Kıtır</t>
         </is>
       </c>
       <c r="D187" s="4" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E187" s="5" t="inlineStr">
         <is>
@@ -6235,7 +6229,7 @@
       </c>
       <c r="H187" s="11" t="inlineStr">
         <is>
-          <t>Acılı Kıtır</t>
+          <t>Zencefilli Kıtır</t>
         </is>
       </c>
     </row>
@@ -6252,11 +6246,11 @@
       </c>
       <c r="C188" s="11" t="inlineStr">
         <is>
-          <t>Haşhaşlı Cips</t>
+          <t>Acılı Kıtır</t>
         </is>
       </c>
       <c r="D188" s="4" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E188" s="5" t="inlineStr">
         <is>
@@ -6266,12 +6260,12 @@
       <c r="F188" s="5" t="n"/>
       <c r="G188" s="9" t="inlineStr">
         <is>
-          <t>Cips</t>
+          <t>Kıtır</t>
         </is>
       </c>
       <c r="H188" s="11" t="inlineStr">
         <is>
-          <t>Haşhaşlı Cips</t>
+          <t>Acılı Kıtır</t>
         </is>
       </c>
     </row>
@@ -6288,11 +6282,11 @@
       </c>
       <c r="C189" s="11" t="inlineStr">
         <is>
-          <t>İrmikli Cips</t>
+          <t>Haşhaşlı Cips</t>
         </is>
       </c>
       <c r="D189" s="4" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E189" s="5" t="inlineStr">
         <is>
@@ -6307,7 +6301,7 @@
       </c>
       <c r="H189" s="11" t="inlineStr">
         <is>
-          <t>İrmikli Cips</t>
+          <t>Haşhaşlı Cips</t>
         </is>
       </c>
     </row>
@@ -6324,11 +6318,11 @@
       </c>
       <c r="C190" s="11" t="inlineStr">
         <is>
-          <t>Parmesanlı Cips</t>
+          <t>İrmikli Cips</t>
         </is>
       </c>
       <c r="D190" s="4" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E190" s="5" t="inlineStr">
         <is>
@@ -6343,7 +6337,7 @@
       </c>
       <c r="H190" s="11" t="inlineStr">
         <is>
-          <t>Parmesanlı Cips</t>
+          <t>İrmikli Cips</t>
         </is>
       </c>
     </row>
@@ -6360,11 +6354,11 @@
       </c>
       <c r="C191" s="11" t="inlineStr">
         <is>
-          <t>Tam Buğday Cips</t>
+          <t>Parmesanlı Cips</t>
         </is>
       </c>
       <c r="D191" s="4" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E191" s="5" t="inlineStr">
         <is>
@@ -6379,67 +6373,71 @@
       </c>
       <c r="H191" s="11" t="inlineStr">
         <is>
+          <t>Parmesanlı Cips</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="11" t="inlineStr">
+        <is>
+          <t>Tuzlu Kurabiye</t>
+        </is>
+      </c>
+      <c r="B192" s="11" t="inlineStr">
+        <is>
+          <t>Galeta / Kıtır / Cips / Diğer Tuzlu</t>
+        </is>
+      </c>
+      <c r="C192" s="11" t="inlineStr">
+        <is>
           <t>Tam Buğday Cips</t>
         </is>
       </c>
-    </row>
-    <row r="192">
-      <c r="A192" s="2" t="inlineStr">
+      <c r="D192" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="E192" s="5" t="inlineStr">
+        <is>
+          <t>tp</t>
+        </is>
+      </c>
+      <c r="F192" s="5" t="n"/>
+      <c r="G192" s="9" t="inlineStr">
+        <is>
+          <t>Cips</t>
+        </is>
+      </c>
+      <c r="H192" s="11" t="inlineStr">
+        <is>
+          <t>Tam Buğday Cips</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="2" t="inlineStr">
         <is>
           <t>Porsiyon Tatlılar</t>
         </is>
       </c>
-      <c r="B192" s="2" t="inlineStr">
+      <c r="B193" s="2" t="inlineStr">
         <is>
           <t>Porsiyon Tatlılar</t>
         </is>
       </c>
-      <c r="C192" s="11" t="inlineStr">
+      <c r="C193" s="11" t="inlineStr">
         <is>
           <t>Tiramisu Dilim</t>
         </is>
       </c>
-      <c r="D192" s="4" t="n">
+      <c r="D193" s="4" t="n">
         <v>1</v>
-      </c>
-      <c r="E192" s="5" t="n"/>
-      <c r="F192" s="5" t="n"/>
-      <c r="G192" s="9" t="n"/>
-      <c r="H192" s="11" t="inlineStr">
-        <is>
-          <t>Tiramisu Dilim</t>
-        </is>
-      </c>
-    </row>
-    <row r="193">
-      <c r="A193" s="11" t="inlineStr">
-        <is>
-          <t>Porsiyon Tatlılar</t>
-        </is>
-      </c>
-      <c r="B193" s="11" t="inlineStr">
-        <is>
-          <t>Porsiyon Tatlılar</t>
-        </is>
-      </c>
-      <c r="C193" s="11" t="inlineStr">
-        <is>
-          <t>Magnolia Çilek</t>
-        </is>
-      </c>
-      <c r="D193" s="4" t="n">
-        <v>2</v>
       </c>
       <c r="E193" s="5" t="n"/>
       <c r="F193" s="5" t="n"/>
-      <c r="G193" s="9" t="inlineStr">
-        <is>
-          <t>Magnolia</t>
-        </is>
-      </c>
+      <c r="G193" s="9" t="n"/>
       <c r="H193" s="11" t="inlineStr">
         <is>
-          <t>Magnolia Çilek</t>
+          <t>Tiramisu Dilim</t>
         </is>
       </c>
     </row>
@@ -6456,11 +6454,11 @@
       </c>
       <c r="C194" s="11" t="inlineStr">
         <is>
-          <t>Magnolia Muzlu</t>
+          <t>Magnolia Çilek</t>
         </is>
       </c>
       <c r="D194" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E194" s="5" t="n"/>
       <c r="F194" s="5" t="n"/>
@@ -6471,7 +6469,7 @@
       </c>
       <c r="H194" s="11" t="inlineStr">
         <is>
-          <t>Magnolia Muzlu</t>
+          <t>Magnolia Çilek</t>
         </is>
       </c>
     </row>
@@ -6488,11 +6486,11 @@
       </c>
       <c r="C195" s="11" t="inlineStr">
         <is>
-          <t>Magnolia Oreolu</t>
+          <t>Magnolia Muzlu</t>
         </is>
       </c>
       <c r="D195" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E195" s="5" t="n"/>
       <c r="F195" s="5" t="n"/>
@@ -6503,7 +6501,7 @@
       </c>
       <c r="H195" s="11" t="inlineStr">
         <is>
-          <t>Magnolia Oreolu</t>
+          <t>Magnolia Muzlu</t>
         </is>
       </c>
     </row>
@@ -6520,11 +6518,11 @@
       </c>
       <c r="C196" s="11" t="inlineStr">
         <is>
-          <t>Dubai Magnolia</t>
+          <t>Magnolia Oreolu</t>
         </is>
       </c>
       <c r="D196" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E196" s="5" t="n"/>
       <c r="F196" s="5" t="n"/>
@@ -6535,7 +6533,7 @@
       </c>
       <c r="H196" s="11" t="inlineStr">
         <is>
-          <t>Dubai Magnolia</t>
+          <t>Magnolia Oreolu</t>
         </is>
       </c>
     </row>
@@ -6552,18 +6550,22 @@
       </c>
       <c r="C197" s="11" t="inlineStr">
         <is>
-          <t>Supangle</t>
+          <t>Dubai Magnolia</t>
         </is>
       </c>
       <c r="D197" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E197" s="5" t="n"/>
       <c r="F197" s="5" t="n"/>
-      <c r="G197" s="9" t="n"/>
+      <c r="G197" s="9" t="inlineStr">
+        <is>
+          <t>Magnolia</t>
+        </is>
+      </c>
       <c r="H197" s="11" t="inlineStr">
         <is>
-          <t>Supangle</t>
+          <t>Dubai Magnolia</t>
         </is>
       </c>
     </row>
@@ -6580,18 +6582,18 @@
       </c>
       <c r="C198" s="11" t="inlineStr">
         <is>
-          <t>Profiterol Kase</t>
+          <t>Supangle</t>
         </is>
       </c>
       <c r="D198" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E198" s="5" t="n"/>
       <c r="F198" s="5" t="n"/>
       <c r="G198" s="9" t="n"/>
       <c r="H198" s="11" t="inlineStr">
         <is>
-          <t>Profiterol Kase</t>
+          <t>Supangle</t>
         </is>
       </c>
     </row>
@@ -6608,18 +6610,18 @@
       </c>
       <c r="C199" s="11" t="inlineStr">
         <is>
-          <t>Mozaik</t>
+          <t>Profiterol Kase</t>
         </is>
       </c>
       <c r="D199" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E199" s="5" t="n"/>
       <c r="F199" s="5" t="n"/>
       <c r="G199" s="9" t="n"/>
       <c r="H199" s="11" t="inlineStr">
         <is>
-          <t>Mozaik</t>
+          <t>Profiterol Kase</t>
         </is>
       </c>
     </row>
@@ -6636,18 +6638,18 @@
       </c>
       <c r="C200" s="11" t="inlineStr">
         <is>
-          <t>Hasbahçe Tek</t>
+          <t>Mozaik</t>
         </is>
       </c>
       <c r="D200" s="4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E200" s="5" t="n"/>
       <c r="F200" s="5" t="n"/>
       <c r="G200" s="9" t="n"/>
       <c r="H200" s="11" t="inlineStr">
         <is>
-          <t>Hasbahçe Tek</t>
+          <t>Mozaik</t>
         </is>
       </c>
     </row>
@@ -6664,18 +6666,18 @@
       </c>
       <c r="C201" s="11" t="inlineStr">
         <is>
-          <t>Fıstıklı Çikolatalı Tek</t>
+          <t>Hasbahçe Tek</t>
         </is>
       </c>
       <c r="D201" s="4" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E201" s="5" t="n"/>
       <c r="F201" s="5" t="n"/>
       <c r="G201" s="9" t="n"/>
       <c r="H201" s="11" t="inlineStr">
         <is>
-          <t>Fıstıklı Çikolatalı Tek</t>
+          <t>Hasbahçe Tek</t>
         </is>
       </c>
     </row>
@@ -6692,18 +6694,18 @@
       </c>
       <c r="C202" s="11" t="inlineStr">
         <is>
-          <t>Kestaneli Tek</t>
+          <t>Fıstıklı Çikolatalı Tek</t>
         </is>
       </c>
       <c r="D202" s="4" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E202" s="5" t="n"/>
       <c r="F202" s="5" t="n"/>
       <c r="G202" s="9" t="n"/>
       <c r="H202" s="11" t="inlineStr">
         <is>
-          <t>Kestaneli Tek</t>
+          <t>Fıstıklı Çikolatalı Tek</t>
         </is>
       </c>
     </row>
@@ -6720,18 +6722,18 @@
       </c>
       <c r="C203" s="11" t="inlineStr">
         <is>
-          <t>Ganaj Tek</t>
+          <t>Kestaneli Tek</t>
         </is>
       </c>
       <c r="D203" s="4" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E203" s="5" t="n"/>
       <c r="F203" s="5" t="n"/>
       <c r="G203" s="9" t="n"/>
       <c r="H203" s="11" t="inlineStr">
         <is>
-          <t>Ganaj Tek</t>
+          <t>Kestaneli Tek</t>
         </is>
       </c>
     </row>
@@ -6748,71 +6750,67 @@
       </c>
       <c r="C204" s="11" t="inlineStr">
         <is>
-          <t>Latte (Porsiyon)</t>
+          <t>Ganaj Tek</t>
         </is>
       </c>
       <c r="D204" s="4" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E204" s="5" t="n"/>
       <c r="F204" s="5" t="n"/>
       <c r="G204" s="9" t="n"/>
       <c r="H204" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Latte </t>
+          <t>Ganaj Tek</t>
         </is>
       </c>
     </row>
     <row r="205">
-      <c r="A205" s="8" t="inlineStr">
+      <c r="A205" s="11" t="inlineStr">
         <is>
           <t>Porsiyon Tatlılar</t>
         </is>
       </c>
-      <c r="B205" s="8" t="inlineStr">
-        <is>
-          <t>Minik Tatlılar</t>
+      <c r="B205" s="11" t="inlineStr">
+        <is>
+          <t>Porsiyon Tatlılar</t>
         </is>
       </c>
       <c r="C205" s="11" t="inlineStr">
         <is>
-          <t>Çikolatalı Ekler (Porsiyon)</t>
+          <t>Latte (Porsiyon)</t>
         </is>
       </c>
       <c r="D205" s="4" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="E205" s="5" t="n"/>
       <c r="F205" s="5" t="n"/>
-      <c r="G205" s="9" t="inlineStr">
-        <is>
-          <t>Ekler</t>
-        </is>
-      </c>
+      <c r="G205" s="9" t="n"/>
       <c r="H205" s="11" t="inlineStr">
         <is>
-          <t>Çikolatalı Ekler (kg)</t>
+          <t xml:space="preserve">Latte </t>
         </is>
       </c>
     </row>
     <row r="206">
-      <c r="A206" s="11" t="inlineStr">
+      <c r="A206" s="8" t="inlineStr">
         <is>
           <t>Porsiyon Tatlılar</t>
         </is>
       </c>
-      <c r="B206" s="11" t="inlineStr">
+      <c r="B206" s="8" t="inlineStr">
         <is>
           <t>Minik Tatlılar</t>
         </is>
       </c>
       <c r="C206" s="11" t="inlineStr">
         <is>
-          <t>Limonlu Ekler (Porsiyon)</t>
+          <t>Çikolatalı Ekler (Porsiyon)</t>
         </is>
       </c>
       <c r="D206" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E206" s="5" t="n"/>
       <c r="F206" s="5" t="n"/>
@@ -6823,7 +6821,7 @@
       </c>
       <c r="H206" s="11" t="inlineStr">
         <is>
-          <t>Limonlu Ekler (kg)</t>
+          <t>Çikolatalı Ekler (kg)</t>
         </is>
       </c>
     </row>
@@ -6840,11 +6838,11 @@
       </c>
       <c r="C207" s="11" t="inlineStr">
         <is>
-          <t>Beyaz Ekler</t>
+          <t>Limonlu Ekler (Porsiyon)</t>
         </is>
       </c>
       <c r="D207" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E207" s="5" t="n"/>
       <c r="F207" s="5" t="n"/>
@@ -6855,7 +6853,7 @@
       </c>
       <c r="H207" s="11" t="inlineStr">
         <is>
-          <t>Beyaz Ekler (kg)</t>
+          <t>Limonlu Ekler (kg)</t>
         </is>
       </c>
     </row>
@@ -6872,22 +6870,22 @@
       </c>
       <c r="C208" s="11" t="inlineStr">
         <is>
-          <t>Petifür</t>
+          <t>Beyaz Ekler</t>
         </is>
       </c>
       <c r="D208" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E208" s="5" t="n"/>
       <c r="F208" s="5" t="n"/>
       <c r="G208" s="9" t="inlineStr">
         <is>
-          <t>Petifür &amp; Rulo</t>
+          <t>Ekler</t>
         </is>
       </c>
       <c r="H208" s="11" t="inlineStr">
         <is>
-          <t>Petifür (kg)</t>
+          <t>Beyaz Ekler (kg)</t>
         </is>
       </c>
     </row>
@@ -6904,11 +6902,11 @@
       </c>
       <c r="C209" s="11" t="inlineStr">
         <is>
-          <t>Rulo Petifür Muzlu</t>
+          <t>Petifür</t>
         </is>
       </c>
       <c r="D209" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E209" s="5" t="n"/>
       <c r="F209" s="5" t="n"/>
@@ -6919,7 +6917,7 @@
       </c>
       <c r="H209" s="11" t="inlineStr">
         <is>
-          <t>Rulo Petifür Muzlu (kg)</t>
+          <t>Petifür (kg)</t>
         </is>
       </c>
     </row>
@@ -6936,11 +6934,11 @@
       </c>
       <c r="C210" s="11" t="inlineStr">
         <is>
-          <t>Rulo Petifür Çilek</t>
+          <t>Rulo Petifür Muzlu</t>
         </is>
       </c>
       <c r="D210" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E210" s="5" t="n"/>
       <c r="F210" s="5" t="n"/>
@@ -6951,7 +6949,7 @@
       </c>
       <c r="H210" s="11" t="inlineStr">
         <is>
-          <t>Rulo Petifür Çilek (kg)</t>
+          <t>Rulo Petifür Muzlu (kg)</t>
         </is>
       </c>
     </row>
@@ -6968,18 +6966,22 @@
       </c>
       <c r="C211" s="11" t="inlineStr">
         <is>
-          <t>Çiko Limon Parfe</t>
+          <t>Rulo Petifür Çilek</t>
         </is>
       </c>
       <c r="D211" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E211" s="5" t="n"/>
       <c r="F211" s="5" t="n"/>
-      <c r="G211" s="9" t="n"/>
+      <c r="G211" s="9" t="inlineStr">
+        <is>
+          <t>Petifür &amp; Rulo</t>
+        </is>
+      </c>
       <c r="H211" s="11" t="inlineStr">
         <is>
-          <t>Çiko Limon Parfe (kg)</t>
+          <t>Rulo Petifür Çilek (kg)</t>
         </is>
       </c>
     </row>
@@ -6996,22 +6998,18 @@
       </c>
       <c r="C212" s="11" t="inlineStr">
         <is>
-          <t>Çilekli Adet Rulo</t>
+          <t>Çiko Limon Parfe</t>
         </is>
       </c>
       <c r="D212" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E212" s="5" t="n"/>
       <c r="F212" s="5" t="n"/>
-      <c r="G212" s="9" t="inlineStr">
-        <is>
-          <t>Petifür &amp; Rulo</t>
-        </is>
-      </c>
+      <c r="G212" s="9" t="n"/>
       <c r="H212" s="11" t="inlineStr">
         <is>
-          <t>Çilekli Adet Rulo</t>
+          <t>Çiko Limon Parfe (kg)</t>
         </is>
       </c>
     </row>
@@ -7028,11 +7026,11 @@
       </c>
       <c r="C213" s="11" t="inlineStr">
         <is>
-          <t>Muzlu Adet Rulo</t>
+          <t>Çilekli Adet Rulo</t>
         </is>
       </c>
       <c r="D213" s="4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E213" s="5" t="n"/>
       <c r="F213" s="5" t="n"/>
@@ -7043,7 +7041,7 @@
       </c>
       <c r="H213" s="11" t="inlineStr">
         <is>
-          <t>Muzlu Adet Rulo</t>
+          <t>Çilekli Adet Rulo</t>
         </is>
       </c>
     </row>
@@ -7060,22 +7058,22 @@
       </c>
       <c r="C214" s="11" t="inlineStr">
         <is>
-          <t>Krokanlı Şu Topu</t>
+          <t>Muzlu Adet Rulo</t>
         </is>
       </c>
       <c r="D214" s="4" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E214" s="5" t="n"/>
       <c r="F214" s="5" t="n"/>
       <c r="G214" s="9" t="inlineStr">
         <is>
-          <t>Şu Topu</t>
+          <t>Petifür &amp; Rulo</t>
         </is>
       </c>
       <c r="H214" s="11" t="inlineStr">
         <is>
-          <t>Krokanlı Şu Topu</t>
+          <t>Muzlu Adet Rulo</t>
         </is>
       </c>
     </row>
@@ -7092,11 +7090,11 @@
       </c>
       <c r="C215" s="11" t="inlineStr">
         <is>
-          <t>Çilekli Şu Topu</t>
+          <t>Krokanlı Şu Topu</t>
         </is>
       </c>
       <c r="D215" s="4" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E215" s="5" t="n"/>
       <c r="F215" s="5" t="n"/>
@@ -7107,63 +7105,67 @@
       </c>
       <c r="H215" s="11" t="inlineStr">
         <is>
+          <t>Krokanlı Şu Topu</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="11" t="inlineStr">
+        <is>
+          <t>Porsiyon Tatlılar</t>
+        </is>
+      </c>
+      <c r="B216" s="11" t="inlineStr">
+        <is>
+          <t>Minik Tatlılar</t>
+        </is>
+      </c>
+      <c r="C216" s="11" t="inlineStr">
+        <is>
           <t>Çilekli Şu Topu</t>
         </is>
       </c>
-    </row>
-    <row r="216">
-      <c r="A216" s="2" t="inlineStr">
-        <is>
-          <t>Porsiyon Tatlılar</t>
-        </is>
-      </c>
-      <c r="B216" s="2" t="inlineStr">
-        <is>
-          <t>Sütlü Tatlı</t>
-        </is>
-      </c>
-      <c r="C216" s="11" t="inlineStr">
-        <is>
-          <t>Kazandibi</t>
-        </is>
-      </c>
       <c r="D216" s="4" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="E216" s="5" t="n"/>
       <c r="F216" s="5" t="n"/>
-      <c r="G216" s="9" t="n"/>
+      <c r="G216" s="9" t="inlineStr">
+        <is>
+          <t>Şu Topu</t>
+        </is>
+      </c>
       <c r="H216" s="11" t="inlineStr">
         <is>
+          <t>Çilekli Şu Topu</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" s="2" t="inlineStr">
+        <is>
+          <t>Porsiyon Tatlılar</t>
+        </is>
+      </c>
+      <c r="B217" s="2" t="inlineStr">
+        <is>
+          <t>Sütlü Tatlı</t>
+        </is>
+      </c>
+      <c r="C217" s="11" t="inlineStr">
+        <is>
           <t>Kazandibi</t>
         </is>
       </c>
-    </row>
-    <row r="217">
-      <c r="A217" s="11" t="inlineStr">
-        <is>
-          <t>Porsiyon Tatlılar</t>
-        </is>
-      </c>
-      <c r="B217" s="11" t="inlineStr">
-        <is>
-          <t>Sütlü Tatlı</t>
-        </is>
-      </c>
-      <c r="C217" s="11" t="inlineStr">
-        <is>
-          <t>Sütlaç</t>
-        </is>
-      </c>
       <c r="D217" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E217" s="5" t="n"/>
       <c r="F217" s="5" t="n"/>
       <c r="G217" s="9" t="n"/>
       <c r="H217" s="11" t="inlineStr">
         <is>
-          <t>Sütlaç</t>
+          <t>Kazandibi</t>
         </is>
       </c>
     </row>
@@ -7180,18 +7182,18 @@
       </c>
       <c r="C218" s="11" t="inlineStr">
         <is>
-          <t>Aşure</t>
+          <t>Sütlaç</t>
         </is>
       </c>
       <c r="D218" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E218" s="5" t="n"/>
       <c r="F218" s="5" t="n"/>
       <c r="G218" s="9" t="n"/>
       <c r="H218" s="11" t="inlineStr">
         <is>
-          <t>Aşure</t>
+          <t>Sütlaç</t>
         </is>
       </c>
     </row>
@@ -7203,27 +7205,23 @@
       </c>
       <c r="B219" s="11" t="inlineStr">
         <is>
-          <t>Porsiyon Tatlılar</t>
+          <t>Sütlü Tatlı</t>
         </is>
       </c>
       <c r="C219" s="11" t="inlineStr">
         <is>
-          <t>Trileçe Frambuaz</t>
+          <t>Aşure</t>
         </is>
       </c>
       <c r="D219" s="4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E219" s="5" t="n"/>
       <c r="F219" s="5" t="n"/>
-      <c r="G219" s="9" t="inlineStr">
-        <is>
-          <t>Trileçe</t>
-        </is>
-      </c>
+      <c r="G219" s="9" t="n"/>
       <c r="H219" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Frambuaz Triliçe</t>
+          <t>Aşure</t>
         </is>
       </c>
     </row>
@@ -7240,11 +7238,11 @@
       </c>
       <c r="C220" s="11" t="inlineStr">
         <is>
-          <t>Trileçe Karamel</t>
+          <t>Trileçe Frambuaz</t>
         </is>
       </c>
       <c r="D220" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E220" s="5" t="n"/>
       <c r="F220" s="5" t="n"/>
@@ -7254,6 +7252,38 @@
         </is>
       </c>
       <c r="H220" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Frambuaz Triliçe</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" s="11" t="inlineStr">
+        <is>
+          <t>Porsiyon Tatlılar</t>
+        </is>
+      </c>
+      <c r="B221" s="11" t="inlineStr">
+        <is>
+          <t>Porsiyon Tatlılar</t>
+        </is>
+      </c>
+      <c r="C221" s="11" t="inlineStr">
+        <is>
+          <t>Trileçe Karamel</t>
+        </is>
+      </c>
+      <c r="D221" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E221" s="5" t="n"/>
+      <c r="F221" s="5" t="n"/>
+      <c r="G221" s="9" t="inlineStr">
+        <is>
+          <t>Trileçe</t>
+        </is>
+      </c>
+      <c r="H221" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve"> Karamel Triliçe</t>
         </is>

</xml_diff>

<commit_message>
Patlıcanlı Sarma'yı Kornet Dereotlu'nun üstüne al, Cevizli Kekikli Sarma ekle
</commit_message>
<xml_diff>
--- a/rapor-duzeni.xlsx
+++ b/rapor-duzeni.xlsx
@@ -500,7 +500,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H221"/>
+  <dimension ref="A1:H222"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4836,32 +4836,34 @@
       </c>
     </row>
     <row r="144">
-      <c r="A144" t="inlineStr">
+      <c r="A144" s="11" t="inlineStr">
         <is>
           <t>Tuzlu Kurabiye</t>
         </is>
       </c>
-      <c r="B144" t="inlineStr">
+      <c r="B144" s="11" t="inlineStr">
         <is>
           <t>Börekli Taş &amp; Poğaça Grubu</t>
         </is>
       </c>
-      <c r="C144" t="inlineStr">
-        <is>
-          <t>Patlıcanlı Sarma</t>
-        </is>
-      </c>
-      <c r="D144" t="n">
+      <c r="C144" s="11" t="inlineStr">
+        <is>
+          <t>Zeytinli</t>
+        </is>
+      </c>
+      <c r="D144" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="E144" t="inlineStr">
+      <c r="E144" s="5" t="inlineStr">
         <is>
           <t>tp</t>
         </is>
       </c>
-      <c r="H144" t="inlineStr">
-        <is>
-          <t>Patlıcanlı Sarma</t>
+      <c r="F144" s="5" t="n"/>
+      <c r="G144" s="9" t="n"/>
+      <c r="H144" s="11" t="inlineStr">
+        <is>
+          <t>Zeytinli</t>
         </is>
       </c>
     </row>
@@ -4878,7 +4880,7 @@
       </c>
       <c r="C145" s="11" t="inlineStr">
         <is>
-          <t>Zeytinli</t>
+          <t>Patatesli</t>
         </is>
       </c>
       <c r="D145" s="4" t="n">
@@ -4893,71 +4895,67 @@
       <c r="G145" s="9" t="n"/>
       <c r="H145" s="11" t="inlineStr">
         <is>
-          <t>Zeytinli</t>
+          <t>Patatesli</t>
         </is>
       </c>
     </row>
     <row r="146">
-      <c r="A146" s="11" t="inlineStr">
+      <c r="A146" t="inlineStr">
         <is>
           <t>Tuzlu Kurabiye</t>
         </is>
       </c>
-      <c r="B146" s="11" t="inlineStr">
+      <c r="B146" t="inlineStr">
         <is>
           <t>Börekli Taş &amp; Poğaça Grubu</t>
         </is>
       </c>
-      <c r="C146" s="11" t="inlineStr">
-        <is>
-          <t>Patatesli</t>
-        </is>
-      </c>
-      <c r="D146" s="4" t="n">
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>Patlıcanlı Sarma</t>
+        </is>
+      </c>
+      <c r="D146" t="n">
         <v>5</v>
       </c>
-      <c r="E146" s="5" t="inlineStr">
+      <c r="E146" t="inlineStr">
         <is>
           <t>tp</t>
         </is>
       </c>
-      <c r="F146" s="5" t="n"/>
-      <c r="G146" s="9" t="n"/>
-      <c r="H146" s="11" t="inlineStr">
-        <is>
-          <t>Patatesli</t>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>Patlıcanlı Sarma</t>
         </is>
       </c>
     </row>
     <row r="147">
-      <c r="A147" s="11" t="inlineStr">
+      <c r="A147" t="inlineStr">
         <is>
           <t>Tuzlu Kurabiye</t>
         </is>
       </c>
-      <c r="B147" s="11" t="inlineStr">
+      <c r="B147" t="inlineStr">
         <is>
           <t>Börekli Taş &amp; Poğaça Grubu</t>
         </is>
       </c>
-      <c r="C147" s="11" t="inlineStr">
-        <is>
-          <t>Kornet Dereotlu</t>
-        </is>
-      </c>
-      <c r="D147" s="4" t="n">
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Cevizli Kekikli Sarma</t>
+        </is>
+      </c>
+      <c r="D147" t="n">
         <v>6</v>
       </c>
-      <c r="E147" s="5" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="F147" s="5" t="n"/>
-      <c r="G147" s="9" t="n"/>
-      <c r="H147" s="11" t="inlineStr">
-        <is>
-          <t>Kornet Dereotlu</t>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>tp</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>Cevizli Kekikli Sarma</t>
         </is>
       </c>
     </row>
@@ -4974,7 +4972,7 @@
       </c>
       <c r="C148" s="11" t="inlineStr">
         <is>
-          <t>Dereotlu Sufle</t>
+          <t>Kornet Dereotlu</t>
         </is>
       </c>
       <c r="D148" s="4" t="n">
@@ -4989,7 +4987,7 @@
       <c r="G148" s="9" t="n"/>
       <c r="H148" s="11" t="inlineStr">
         <is>
-          <t>Dereotlu Sufle</t>
+          <t>Kornet Dereotlu</t>
         </is>
       </c>
     </row>
@@ -5006,7 +5004,7 @@
       </c>
       <c r="C149" s="11" t="inlineStr">
         <is>
-          <t>Sebzeli</t>
+          <t>Dereotlu Sufle</t>
         </is>
       </c>
       <c r="D149" s="4" t="n">
@@ -5014,14 +5012,14 @@
       </c>
       <c r="E149" s="5" t="inlineStr">
         <is>
-          <t>tp</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="F149" s="5" t="n"/>
       <c r="G149" s="9" t="n"/>
       <c r="H149" s="11" t="inlineStr">
         <is>
-          <t>Sebzeli</t>
+          <t>Dereotlu Sufle</t>
         </is>
       </c>
     </row>
@@ -5038,7 +5036,7 @@
       </c>
       <c r="C150" s="11" t="inlineStr">
         <is>
-          <t>Patlıcanlı</t>
+          <t>Sebzeli</t>
         </is>
       </c>
       <c r="D150" s="4" t="n">
@@ -5053,7 +5051,7 @@
       <c r="G150" s="9" t="n"/>
       <c r="H150" s="11" t="inlineStr">
         <is>
-          <t>Patlıcanlı</t>
+          <t>Sebzeli</t>
         </is>
       </c>
     </row>
@@ -5070,7 +5068,7 @@
       </c>
       <c r="C151" s="11" t="inlineStr">
         <is>
-          <t>Mini Pizza</t>
+          <t>Patlıcanlı</t>
         </is>
       </c>
       <c r="D151" s="4" t="n">
@@ -5085,7 +5083,7 @@
       <c r="G151" s="9" t="n"/>
       <c r="H151" s="11" t="inlineStr">
         <is>
-          <t>Mini Pizza</t>
+          <t>Patlıcanlı</t>
         </is>
       </c>
     </row>
@@ -5102,7 +5100,7 @@
       </c>
       <c r="C152" s="11" t="inlineStr">
         <is>
-          <t>Minik Simit</t>
+          <t>Mini Pizza</t>
         </is>
       </c>
       <c r="D152" s="4" t="n">
@@ -5117,7 +5115,7 @@
       <c r="G152" s="9" t="n"/>
       <c r="H152" s="11" t="inlineStr">
         <is>
-          <t>Minik Simit</t>
+          <t>Mini Pizza</t>
         </is>
       </c>
     </row>
@@ -5134,7 +5132,7 @@
       </c>
       <c r="C153" s="11" t="inlineStr">
         <is>
-          <t>Düz Örgü</t>
+          <t>Minik Simit</t>
         </is>
       </c>
       <c r="D153" s="4" t="n">
@@ -5149,7 +5147,7 @@
       <c r="G153" s="9" t="n"/>
       <c r="H153" s="11" t="inlineStr">
         <is>
-          <t>Düz Örgü</t>
+          <t>Minik Simit</t>
         </is>
       </c>
     </row>
@@ -5166,7 +5164,7 @@
       </c>
       <c r="C154" s="11" t="inlineStr">
         <is>
-          <t>Yuvarlak Örgü</t>
+          <t>Düz Örgü</t>
         </is>
       </c>
       <c r="D154" s="4" t="n">
@@ -5181,7 +5179,7 @@
       <c r="G154" s="9" t="n"/>
       <c r="H154" s="11" t="inlineStr">
         <is>
-          <t>Yuvarlak Örgü</t>
+          <t>Düz Örgü</t>
         </is>
       </c>
     </row>
@@ -5198,7 +5196,7 @@
       </c>
       <c r="C155" s="11" t="inlineStr">
         <is>
-          <t>Burgu Susamlı Haşhaşlı</t>
+          <t>Yuvarlak Örgü</t>
         </is>
       </c>
       <c r="D155" s="4" t="n">
@@ -5213,67 +5211,67 @@
       <c r="G155" s="9" t="n"/>
       <c r="H155" s="11" t="inlineStr">
         <is>
+          <t>Yuvarlak Örgü</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="11" t="inlineStr">
+        <is>
+          <t>Tuzlu Kurabiye</t>
+        </is>
+      </c>
+      <c r="B156" s="11" t="inlineStr">
+        <is>
+          <t>Börekli Taş &amp; Poğaça Grubu</t>
+        </is>
+      </c>
+      <c r="C156" s="11" t="inlineStr">
+        <is>
           <t>Burgu Susamlı Haşhaşlı</t>
         </is>
       </c>
-    </row>
-    <row r="156">
-      <c r="A156" s="2" t="inlineStr">
-        <is>
-          <t>Tuzlu Kurabiye</t>
-        </is>
-      </c>
-      <c r="B156" s="2" t="inlineStr">
-        <is>
-          <t>Diyet Kurabiyeler</t>
-        </is>
-      </c>
-      <c r="C156" s="11" t="inlineStr">
-        <is>
-          <t>Burgu Tahıllı</t>
-        </is>
-      </c>
       <c r="D156" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E156" s="5" t="n"/>
+        <v>15</v>
+      </c>
+      <c r="E156" s="5" t="inlineStr">
+        <is>
+          <t>tp</t>
+        </is>
+      </c>
       <c r="F156" s="5" t="n"/>
       <c r="G156" s="9" t="n"/>
       <c r="H156" s="11" t="inlineStr">
         <is>
+          <t>Burgu Susamlı Haşhaşlı</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="2" t="inlineStr">
+        <is>
+          <t>Tuzlu Kurabiye</t>
+        </is>
+      </c>
+      <c r="B157" s="2" t="inlineStr">
+        <is>
+          <t>Diyet Kurabiyeler</t>
+        </is>
+      </c>
+      <c r="C157" s="11" t="inlineStr">
+        <is>
           <t>Burgu Tahıllı</t>
         </is>
       </c>
-    </row>
-    <row r="157">
-      <c r="A157" s="11" t="inlineStr">
-        <is>
-          <t>Tuzlu Kurabiye</t>
-        </is>
-      </c>
-      <c r="B157" s="11" t="inlineStr">
-        <is>
-          <t>Diyet Kurabiyeler</t>
-        </is>
-      </c>
-      <c r="C157" s="11" t="inlineStr">
-        <is>
-          <t>Ayçekirdekli Galeta</t>
-        </is>
-      </c>
       <c r="D157" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="E157" s="5" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="E157" s="5" t="n"/>
       <c r="F157" s="5" t="n"/>
       <c r="G157" s="9" t="n"/>
       <c r="H157" s="11" t="inlineStr">
         <is>
-          <t>Ayçekirdekli Galeta</t>
+          <t>Burgu Tahıllı</t>
         </is>
       </c>
     </row>
@@ -5290,22 +5288,22 @@
       </c>
       <c r="C158" s="11" t="inlineStr">
         <is>
-          <t>Parmesan Galeta</t>
+          <t>Ayçekirdekli Galeta</t>
         </is>
       </c>
       <c r="D158" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E158" s="5" t="inlineStr">
         <is>
-          <t>tp</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="F158" s="5" t="n"/>
       <c r="G158" s="9" t="n"/>
       <c r="H158" s="11" t="inlineStr">
         <is>
-          <t>Parmesan Galeta</t>
+          <t>Ayçekirdekli Galeta</t>
         </is>
       </c>
     </row>
@@ -5322,11 +5320,11 @@
       </c>
       <c r="C159" s="11" t="inlineStr">
         <is>
-          <t>İtalyan Galeta</t>
+          <t>Parmesan Galeta</t>
         </is>
       </c>
       <c r="D159" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E159" s="5" t="inlineStr">
         <is>
@@ -5337,7 +5335,7 @@
       <c r="G159" s="9" t="n"/>
       <c r="H159" s="11" t="inlineStr">
         <is>
-          <t>İtalyan Galeta</t>
+          <t>Parmesan Galeta</t>
         </is>
       </c>
     </row>
@@ -5354,11 +5352,11 @@
       </c>
       <c r="C160" s="11" t="inlineStr">
         <is>
-          <t>Biberiyeli Zeytinli Galeta</t>
+          <t>İtalyan Galeta</t>
         </is>
       </c>
       <c r="D160" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E160" s="5" t="inlineStr">
         <is>
@@ -5369,7 +5367,7 @@
       <c r="G160" s="9" t="n"/>
       <c r="H160" s="11" t="inlineStr">
         <is>
-          <t>Biberiyeli Zeytinli Galeta</t>
+          <t>İtalyan Galeta</t>
         </is>
       </c>
     </row>
@@ -5386,11 +5384,11 @@
       </c>
       <c r="C161" s="11" t="inlineStr">
         <is>
-          <t>Çekirdekli Kokteyl</t>
+          <t>Biberiyeli Zeytinli Galeta</t>
         </is>
       </c>
       <c r="D161" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E161" s="5" t="inlineStr">
         <is>
@@ -5401,7 +5399,7 @@
       <c r="G161" s="9" t="n"/>
       <c r="H161" s="11" t="inlineStr">
         <is>
-          <t>Çekirdekli Kokteyl</t>
+          <t>Biberiyeli Zeytinli Galeta</t>
         </is>
       </c>
     </row>
@@ -5418,11 +5416,11 @@
       </c>
       <c r="C162" s="11" t="inlineStr">
         <is>
-          <t>Üzümlü Kepekli</t>
+          <t>Çekirdekli Kokteyl</t>
         </is>
       </c>
       <c r="D162" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E162" s="5" t="inlineStr">
         <is>
@@ -5433,7 +5431,7 @@
       <c r="G162" s="9" t="n"/>
       <c r="H162" s="11" t="inlineStr">
         <is>
-          <t>Üzümlü Kepekli</t>
+          <t>Çekirdekli Kokteyl</t>
         </is>
       </c>
     </row>
@@ -5450,11 +5448,11 @@
       </c>
       <c r="C163" s="11" t="inlineStr">
         <is>
-          <t>Üzümlü Cevizli Kepekli</t>
+          <t>Üzümlü Kepekli</t>
         </is>
       </c>
       <c r="D163" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E163" s="5" t="inlineStr">
         <is>
@@ -5465,7 +5463,7 @@
       <c r="G163" s="9" t="n"/>
       <c r="H163" s="11" t="inlineStr">
         <is>
-          <t>Üzümlü Cevizli Kepekli</t>
+          <t>Üzümlü Kepekli</t>
         </is>
       </c>
     </row>
@@ -5482,18 +5480,22 @@
       </c>
       <c r="C164" s="11" t="inlineStr">
         <is>
-          <t>Kuru Üzümlü Yassı Tahıllı</t>
+          <t>Üzümlü Cevizli Kepekli</t>
         </is>
       </c>
       <c r="D164" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="E164" s="5" t="n"/>
+        <v>8</v>
+      </c>
+      <c r="E164" s="5" t="inlineStr">
+        <is>
+          <t>tp</t>
+        </is>
+      </c>
       <c r="F164" s="5" t="n"/>
       <c r="G164" s="9" t="n"/>
       <c r="H164" s="11" t="inlineStr">
         <is>
-          <t>Kuru Üzümlü Yassı Tahıllı</t>
+          <t>Üzümlü Cevizli Kepekli</t>
         </is>
       </c>
     </row>
@@ -5510,22 +5512,18 @@
       </c>
       <c r="C165" s="11" t="inlineStr">
         <is>
-          <t>Granola Bar Tepsi</t>
+          <t>Kuru Üzümlü Yassı Tahıllı</t>
         </is>
       </c>
       <c r="D165" s="4" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E165" s="5" t="n"/>
       <c r="F165" s="5" t="n"/>
-      <c r="G165" s="9" t="inlineStr">
-        <is>
-          <t>Bar</t>
-        </is>
-      </c>
+      <c r="G165" s="9" t="n"/>
       <c r="H165" s="11" t="inlineStr">
         <is>
-          <t>Granola Bar Tepsi</t>
+          <t>Kuru Üzümlü Yassı Tahıllı</t>
         </is>
       </c>
     </row>
@@ -5542,18 +5540,22 @@
       </c>
       <c r="C166" s="11" t="inlineStr">
         <is>
-          <t>Tahinli Susamlı</t>
+          <t>Granola Bar Tepsi</t>
         </is>
       </c>
       <c r="D166" s="4" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E166" s="5" t="n"/>
       <c r="F166" s="5" t="n"/>
-      <c r="G166" s="9" t="n"/>
+      <c r="G166" s="9" t="inlineStr">
+        <is>
+          <t>Bar</t>
+        </is>
+      </c>
       <c r="H166" s="11" t="inlineStr">
         <is>
-          <t>Tahinli Susamlı</t>
+          <t>Granola Bar Tepsi</t>
         </is>
       </c>
     </row>
@@ -5570,18 +5572,18 @@
       </c>
       <c r="C167" s="11" t="inlineStr">
         <is>
-          <t>Granola Dökme</t>
+          <t>Tahinli Susamlı</t>
         </is>
       </c>
       <c r="D167" s="4" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E167" s="5" t="n"/>
       <c r="F167" s="5" t="n"/>
       <c r="G167" s="9" t="n"/>
       <c r="H167" s="11" t="inlineStr">
         <is>
-          <t>Granola Dökme</t>
+          <t>Tahinli Susamlı</t>
         </is>
       </c>
     </row>
@@ -5598,74 +5600,74 @@
       </c>
       <c r="C168" s="11" t="inlineStr">
         <is>
-          <t>Kalp Denge Tahıllı</t>
+          <t>Granola Dökme</t>
         </is>
       </c>
       <c r="D168" s="4" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E168" s="5" t="n"/>
       <c r="F168" s="5" t="n"/>
       <c r="G168" s="9" t="n"/>
       <c r="H168" s="11" t="inlineStr">
         <is>
+          <t>Granola Dökme</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="11" t="inlineStr">
+        <is>
+          <t>Tuzlu Kurabiye</t>
+        </is>
+      </c>
+      <c r="B169" s="11" t="inlineStr">
+        <is>
+          <t>Diyet Kurabiyeler</t>
+        </is>
+      </c>
+      <c r="C169" s="11" t="inlineStr">
+        <is>
           <t>Kalp Denge Tahıllı</t>
         </is>
       </c>
-    </row>
-    <row r="169">
-      <c r="A169" s="2" t="inlineStr">
-        <is>
-          <t>Tuzlu Kurabiye</t>
-        </is>
-      </c>
-      <c r="B169" s="2" t="inlineStr">
-        <is>
-          <t>Adet Ürünler</t>
-        </is>
-      </c>
-      <c r="C169" s="11" t="inlineStr">
-        <is>
-          <t>Paskalya</t>
-        </is>
-      </c>
       <c r="D169" s="4" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="E169" s="5" t="n"/>
       <c r="F169" s="5" t="n"/>
       <c r="G169" s="9" t="n"/>
       <c r="H169" s="11" t="inlineStr">
         <is>
+          <t>Kalp Denge Tahıllı</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="2" t="inlineStr">
+        <is>
+          <t>Tuzlu Kurabiye</t>
+        </is>
+      </c>
+      <c r="B170" s="2" t="inlineStr">
+        <is>
+          <t>Adet Ürünler</t>
+        </is>
+      </c>
+      <c r="C170" s="11" t="inlineStr">
+        <is>
           <t>Paskalya</t>
         </is>
       </c>
-    </row>
-    <row r="170">
-      <c r="A170" s="11" t="inlineStr">
-        <is>
-          <t>Tuzlu Kurabiye</t>
-        </is>
-      </c>
-      <c r="B170" s="11" t="inlineStr">
-        <is>
-          <t>Adet Ürünler</t>
-        </is>
-      </c>
-      <c r="C170" s="11" t="inlineStr">
-        <is>
-          <t>Paskalya Çikolatalı</t>
-        </is>
-      </c>
       <c r="D170" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E170" s="5" t="n"/>
       <c r="F170" s="5" t="n"/>
       <c r="G170" s="9" t="n"/>
       <c r="H170" s="11" t="inlineStr">
         <is>
-          <t>Paskalya Çikolatalı</t>
+          <t>Paskalya</t>
         </is>
       </c>
     </row>
@@ -5682,18 +5684,18 @@
       </c>
       <c r="C171" s="11" t="inlineStr">
         <is>
-          <t>Tahinli Çörek</t>
+          <t>Paskalya Çikolatalı</t>
         </is>
       </c>
       <c r="D171" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E171" s="5" t="n"/>
       <c r="F171" s="5" t="n"/>
       <c r="G171" s="9" t="n"/>
       <c r="H171" s="11" t="inlineStr">
         <is>
-          <t>Tahinli Çörek</t>
+          <t>Paskalya Çikolatalı</t>
         </is>
       </c>
     </row>
@@ -5710,22 +5712,18 @@
       </c>
       <c r="C172" s="11" t="inlineStr">
         <is>
-          <t>Beze Büyük</t>
+          <t>Tahinli Çörek</t>
         </is>
       </c>
       <c r="D172" s="4" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E172" s="5" t="n"/>
       <c r="F172" s="5" t="n"/>
-      <c r="G172" s="9" t="inlineStr">
-        <is>
-          <t>Beze</t>
-        </is>
-      </c>
+      <c r="G172" s="9" t="n"/>
       <c r="H172" s="11" t="inlineStr">
         <is>
-          <t>Beze Büyük</t>
+          <t>Tahinli Çörek</t>
         </is>
       </c>
     </row>
@@ -5742,11 +5740,11 @@
       </c>
       <c r="C173" s="11" t="inlineStr">
         <is>
-          <t>Beze Beyaz Minik</t>
+          <t>Beze Büyük</t>
         </is>
       </c>
       <c r="D173" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E173" s="5" t="n"/>
       <c r="F173" s="5" t="n"/>
@@ -5757,7 +5755,7 @@
       </c>
       <c r="H173" s="11" t="inlineStr">
         <is>
-          <t>Beze Beyaz Minik</t>
+          <t>Beze Büyük</t>
         </is>
       </c>
     </row>
@@ -5774,11 +5772,11 @@
       </c>
       <c r="C174" s="11" t="inlineStr">
         <is>
-          <t>Beze Renkli Minik</t>
+          <t>Beze Beyaz Minik</t>
         </is>
       </c>
       <c r="D174" s="4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E174" s="5" t="n"/>
       <c r="F174" s="5" t="n"/>
@@ -5789,7 +5787,7 @@
       </c>
       <c r="H174" s="11" t="inlineStr">
         <is>
-          <t>Beze Renkli Minik</t>
+          <t>Beze Beyaz Minik</t>
         </is>
       </c>
     </row>
@@ -5806,18 +5804,22 @@
       </c>
       <c r="C175" s="11" t="inlineStr">
         <is>
-          <t>Acıbadem</t>
+          <t>Beze Renkli Minik</t>
         </is>
       </c>
       <c r="D175" s="4" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="E175" s="5" t="n"/>
       <c r="F175" s="5" t="n"/>
-      <c r="G175" s="9" t="n"/>
+      <c r="G175" s="9" t="inlineStr">
+        <is>
+          <t>Beze</t>
+        </is>
+      </c>
       <c r="H175" s="11" t="inlineStr">
         <is>
-          <t>Acıbadem</t>
+          <t>Beze Renkli Minik</t>
         </is>
       </c>
     </row>
@@ -5834,18 +5836,18 @@
       </c>
       <c r="C176" s="11" t="inlineStr">
         <is>
-          <t>Acıbadem Minik</t>
+          <t>Acıbadem</t>
         </is>
       </c>
       <c r="D176" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E176" s="5" t="n"/>
       <c r="F176" s="5" t="n"/>
       <c r="G176" s="9" t="n"/>
       <c r="H176" s="11" t="inlineStr">
         <is>
-          <t>Acıbadem Minik</t>
+          <t>Acıbadem</t>
         </is>
       </c>
     </row>
@@ -5862,75 +5864,67 @@
       </c>
       <c r="C177" s="11" t="inlineStr">
         <is>
-          <t>Ayçöreği</t>
+          <t>Acıbadem Minik</t>
         </is>
       </c>
       <c r="D177" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E177" s="5" t="n"/>
       <c r="F177" s="5" t="n"/>
       <c r="G177" s="9" t="n"/>
       <c r="H177" s="11" t="inlineStr">
         <is>
+          <t>Acıbadem Minik</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="11" t="inlineStr">
+        <is>
+          <t>Tuzlu Kurabiye</t>
+        </is>
+      </c>
+      <c r="B178" s="11" t="inlineStr">
+        <is>
+          <t>Adet Ürünler</t>
+        </is>
+      </c>
+      <c r="C178" s="11" t="inlineStr">
+        <is>
           <t>Ayçöreği</t>
         </is>
       </c>
-    </row>
-    <row r="178">
-      <c r="A178" s="2" t="inlineStr">
+      <c r="D178" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="E178" s="5" t="n"/>
+      <c r="F178" s="5" t="n"/>
+      <c r="G178" s="9" t="n"/>
+      <c r="H178" s="11" t="inlineStr">
+        <is>
+          <t>Ayçöreği</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="2" t="inlineStr">
         <is>
           <t>Tuzlu Kurabiye</t>
         </is>
       </c>
-      <c r="B178" s="2" t="inlineStr">
+      <c r="B179" s="2" t="inlineStr">
         <is>
           <t>Galeta / Kıtır / Cips / Diğer Tuzlu</t>
         </is>
       </c>
-      <c r="C178" s="11" t="inlineStr">
+      <c r="C179" s="11" t="inlineStr">
         <is>
           <t>Batonsale Sade</t>
         </is>
       </c>
-      <c r="D178" s="4" t="n">
+      <c r="D179" s="4" t="n">
         <v>1</v>
-      </c>
-      <c r="E178" s="5" t="inlineStr">
-        <is>
-          <t>tp</t>
-        </is>
-      </c>
-      <c r="F178" s="5" t="n"/>
-      <c r="G178" s="9" t="inlineStr">
-        <is>
-          <t>Batonsale</t>
-        </is>
-      </c>
-      <c r="H178" s="11" t="inlineStr">
-        <is>
-          <t>Batonsale Sade</t>
-        </is>
-      </c>
-    </row>
-    <row r="179">
-      <c r="A179" s="11" t="inlineStr">
-        <is>
-          <t>Tuzlu Kurabiye</t>
-        </is>
-      </c>
-      <c r="B179" s="11" t="inlineStr">
-        <is>
-          <t>Galeta / Kıtır / Cips / Diğer Tuzlu</t>
-        </is>
-      </c>
-      <c r="C179" s="11" t="inlineStr">
-        <is>
-          <t>Batonsale Çörekotlu</t>
-        </is>
-      </c>
-      <c r="D179" s="4" t="n">
-        <v>2</v>
       </c>
       <c r="E179" s="5" t="inlineStr">
         <is>
@@ -5945,7 +5939,7 @@
       </c>
       <c r="H179" s="11" t="inlineStr">
         <is>
-          <t>Batonsale Çörekotlu</t>
+          <t>Batonsale Sade</t>
         </is>
       </c>
     </row>
@@ -5962,11 +5956,11 @@
       </c>
       <c r="C180" s="11" t="inlineStr">
         <is>
-          <t>Batonsale Kaşarlı</t>
+          <t>Batonsale Çörekotlu</t>
         </is>
       </c>
       <c r="D180" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E180" s="5" t="inlineStr">
         <is>
@@ -5981,7 +5975,7 @@
       </c>
       <c r="H180" s="11" t="inlineStr">
         <is>
-          <t>Batonsale Kaşarlı</t>
+          <t>Batonsale Çörekotlu</t>
         </is>
       </c>
     </row>
@@ -5998,11 +5992,11 @@
       </c>
       <c r="C181" s="11" t="inlineStr">
         <is>
-          <t>Kırık Kırak Susamlı</t>
+          <t>Batonsale Kaşarlı</t>
         </is>
       </c>
       <c r="D181" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E181" s="5" t="inlineStr">
         <is>
@@ -6010,10 +6004,14 @@
         </is>
       </c>
       <c r="F181" s="5" t="n"/>
-      <c r="G181" s="9" t="n"/>
+      <c r="G181" s="9" t="inlineStr">
+        <is>
+          <t>Batonsale</t>
+        </is>
+      </c>
       <c r="H181" s="11" t="inlineStr">
         <is>
-          <t>Kırık Kırak Susamlı</t>
+          <t>Batonsale Kaşarlı</t>
         </is>
       </c>
     </row>
@@ -6030,11 +6028,11 @@
       </c>
       <c r="C182" s="11" t="inlineStr">
         <is>
-          <t>Galet Kaşarlı</t>
+          <t>Kırık Kırak Susamlı</t>
         </is>
       </c>
       <c r="D182" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E182" s="5" t="inlineStr">
         <is>
@@ -6042,14 +6040,10 @@
         </is>
       </c>
       <c r="F182" s="5" t="n"/>
-      <c r="G182" s="9" t="inlineStr">
-        <is>
-          <t>Galet</t>
-        </is>
-      </c>
+      <c r="G182" s="9" t="n"/>
       <c r="H182" s="11" t="inlineStr">
         <is>
-          <t>Galet Kaşarlı</t>
+          <t>Kırık Kırak Susamlı</t>
         </is>
       </c>
     </row>
@@ -6066,11 +6060,11 @@
       </c>
       <c r="C183" s="11" t="inlineStr">
         <is>
-          <t>Galet Çörekotlu</t>
+          <t>Galet Kaşarlı</t>
         </is>
       </c>
       <c r="D183" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E183" s="5" t="inlineStr">
         <is>
@@ -6085,7 +6079,7 @@
       </c>
       <c r="H183" s="11" t="inlineStr">
         <is>
-          <t>Galet Çörekotlu</t>
+          <t>Galet Kaşarlı</t>
         </is>
       </c>
     </row>
@@ -6102,11 +6096,11 @@
       </c>
       <c r="C184" s="11" t="inlineStr">
         <is>
-          <t>Galet Susamlı</t>
+          <t>Galet Çörekotlu</t>
         </is>
       </c>
       <c r="D184" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E184" s="5" t="inlineStr">
         <is>
@@ -6121,7 +6115,7 @@
       </c>
       <c r="H184" s="11" t="inlineStr">
         <is>
-          <t>Galet Susamlı</t>
+          <t>Galet Çörekotlu</t>
         </is>
       </c>
     </row>
@@ -6138,11 +6132,11 @@
       </c>
       <c r="C185" s="11" t="inlineStr">
         <is>
-          <t>Baharatlı Kıtır</t>
+          <t>Galet Susamlı</t>
         </is>
       </c>
       <c r="D185" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E185" s="5" t="inlineStr">
         <is>
@@ -6152,12 +6146,12 @@
       <c r="F185" s="5" t="n"/>
       <c r="G185" s="9" t="inlineStr">
         <is>
-          <t>Kıtır</t>
+          <t>Galet</t>
         </is>
       </c>
       <c r="H185" s="11" t="inlineStr">
         <is>
-          <t>Baharatlı Kıtır</t>
+          <t>Galet Susamlı</t>
         </is>
       </c>
     </row>
@@ -6174,11 +6168,11 @@
       </c>
       <c r="C186" s="11" t="inlineStr">
         <is>
-          <t>Kaşarlı Kıtır</t>
+          <t>Baharatlı Kıtır</t>
         </is>
       </c>
       <c r="D186" s="4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E186" s="5" t="inlineStr">
         <is>
@@ -6193,7 +6187,7 @@
       </c>
       <c r="H186" s="11" t="inlineStr">
         <is>
-          <t>Kaşarlı Kıtır</t>
+          <t>Baharatlı Kıtır</t>
         </is>
       </c>
     </row>
@@ -6210,11 +6204,11 @@
       </c>
       <c r="C187" s="11" t="inlineStr">
         <is>
-          <t>Zencefilli Kıtır</t>
+          <t>Kaşarlı Kıtır</t>
         </is>
       </c>
       <c r="D187" s="4" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E187" s="5" t="inlineStr">
         <is>
@@ -6229,7 +6223,7 @@
       </c>
       <c r="H187" s="11" t="inlineStr">
         <is>
-          <t>Zencefilli Kıtır</t>
+          <t>Kaşarlı Kıtır</t>
         </is>
       </c>
     </row>
@@ -6246,11 +6240,11 @@
       </c>
       <c r="C188" s="11" t="inlineStr">
         <is>
-          <t>Acılı Kıtır</t>
+          <t>Zencefilli Kıtır</t>
         </is>
       </c>
       <c r="D188" s="4" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E188" s="5" t="inlineStr">
         <is>
@@ -6265,7 +6259,7 @@
       </c>
       <c r="H188" s="11" t="inlineStr">
         <is>
-          <t>Acılı Kıtır</t>
+          <t>Zencefilli Kıtır</t>
         </is>
       </c>
     </row>
@@ -6282,11 +6276,11 @@
       </c>
       <c r="C189" s="11" t="inlineStr">
         <is>
-          <t>Haşhaşlı Cips</t>
+          <t>Acılı Kıtır</t>
         </is>
       </c>
       <c r="D189" s="4" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E189" s="5" t="inlineStr">
         <is>
@@ -6296,12 +6290,12 @@
       <c r="F189" s="5" t="n"/>
       <c r="G189" s="9" t="inlineStr">
         <is>
-          <t>Cips</t>
+          <t>Kıtır</t>
         </is>
       </c>
       <c r="H189" s="11" t="inlineStr">
         <is>
-          <t>Haşhaşlı Cips</t>
+          <t>Acılı Kıtır</t>
         </is>
       </c>
     </row>
@@ -6318,11 +6312,11 @@
       </c>
       <c r="C190" s="11" t="inlineStr">
         <is>
-          <t>İrmikli Cips</t>
+          <t>Haşhaşlı Cips</t>
         </is>
       </c>
       <c r="D190" s="4" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E190" s="5" t="inlineStr">
         <is>
@@ -6337,7 +6331,7 @@
       </c>
       <c r="H190" s="11" t="inlineStr">
         <is>
-          <t>İrmikli Cips</t>
+          <t>Haşhaşlı Cips</t>
         </is>
       </c>
     </row>
@@ -6354,11 +6348,11 @@
       </c>
       <c r="C191" s="11" t="inlineStr">
         <is>
-          <t>Parmesanlı Cips</t>
+          <t>İrmikli Cips</t>
         </is>
       </c>
       <c r="D191" s="4" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E191" s="5" t="inlineStr">
         <is>
@@ -6373,7 +6367,7 @@
       </c>
       <c r="H191" s="11" t="inlineStr">
         <is>
-          <t>Parmesanlı Cips</t>
+          <t>İrmikli Cips</t>
         </is>
       </c>
     </row>
@@ -6390,11 +6384,11 @@
       </c>
       <c r="C192" s="11" t="inlineStr">
         <is>
-          <t>Tam Buğday Cips</t>
+          <t>Parmesanlı Cips</t>
         </is>
       </c>
       <c r="D192" s="4" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E192" s="5" t="inlineStr">
         <is>
@@ -6409,67 +6403,71 @@
       </c>
       <c r="H192" s="11" t="inlineStr">
         <is>
+          <t>Parmesanlı Cips</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="11" t="inlineStr">
+        <is>
+          <t>Tuzlu Kurabiye</t>
+        </is>
+      </c>
+      <c r="B193" s="11" t="inlineStr">
+        <is>
+          <t>Galeta / Kıtır / Cips / Diğer Tuzlu</t>
+        </is>
+      </c>
+      <c r="C193" s="11" t="inlineStr">
+        <is>
           <t>Tam Buğday Cips</t>
         </is>
       </c>
-    </row>
-    <row r="193">
-      <c r="A193" s="2" t="inlineStr">
+      <c r="D193" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="E193" s="5" t="inlineStr">
+        <is>
+          <t>tp</t>
+        </is>
+      </c>
+      <c r="F193" s="5" t="n"/>
+      <c r="G193" s="9" t="inlineStr">
+        <is>
+          <t>Cips</t>
+        </is>
+      </c>
+      <c r="H193" s="11" t="inlineStr">
+        <is>
+          <t>Tam Buğday Cips</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="2" t="inlineStr">
         <is>
           <t>Porsiyon Tatlılar</t>
         </is>
       </c>
-      <c r="B193" s="2" t="inlineStr">
+      <c r="B194" s="2" t="inlineStr">
         <is>
           <t>Porsiyon Tatlılar</t>
         </is>
       </c>
-      <c r="C193" s="11" t="inlineStr">
+      <c r="C194" s="11" t="inlineStr">
         <is>
           <t>Tiramisu Dilim</t>
         </is>
       </c>
-      <c r="D193" s="4" t="n">
+      <c r="D194" s="4" t="n">
         <v>1</v>
-      </c>
-      <c r="E193" s="5" t="n"/>
-      <c r="F193" s="5" t="n"/>
-      <c r="G193" s="9" t="n"/>
-      <c r="H193" s="11" t="inlineStr">
-        <is>
-          <t>Tiramisu Dilim</t>
-        </is>
-      </c>
-    </row>
-    <row r="194">
-      <c r="A194" s="11" t="inlineStr">
-        <is>
-          <t>Porsiyon Tatlılar</t>
-        </is>
-      </c>
-      <c r="B194" s="11" t="inlineStr">
-        <is>
-          <t>Porsiyon Tatlılar</t>
-        </is>
-      </c>
-      <c r="C194" s="11" t="inlineStr">
-        <is>
-          <t>Magnolia Çilek</t>
-        </is>
-      </c>
-      <c r="D194" s="4" t="n">
-        <v>2</v>
       </c>
       <c r="E194" s="5" t="n"/>
       <c r="F194" s="5" t="n"/>
-      <c r="G194" s="9" t="inlineStr">
-        <is>
-          <t>Magnolia</t>
-        </is>
-      </c>
+      <c r="G194" s="9" t="n"/>
       <c r="H194" s="11" t="inlineStr">
         <is>
-          <t>Magnolia Çilek</t>
+          <t>Tiramisu Dilim</t>
         </is>
       </c>
     </row>
@@ -6486,11 +6484,11 @@
       </c>
       <c r="C195" s="11" t="inlineStr">
         <is>
-          <t>Magnolia Muzlu</t>
+          <t>Magnolia Çilek</t>
         </is>
       </c>
       <c r="D195" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E195" s="5" t="n"/>
       <c r="F195" s="5" t="n"/>
@@ -6501,7 +6499,7 @@
       </c>
       <c r="H195" s="11" t="inlineStr">
         <is>
-          <t>Magnolia Muzlu</t>
+          <t>Magnolia Çilek</t>
         </is>
       </c>
     </row>
@@ -6518,11 +6516,11 @@
       </c>
       <c r="C196" s="11" t="inlineStr">
         <is>
-          <t>Magnolia Oreolu</t>
+          <t>Magnolia Muzlu</t>
         </is>
       </c>
       <c r="D196" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E196" s="5" t="n"/>
       <c r="F196" s="5" t="n"/>
@@ -6533,7 +6531,7 @@
       </c>
       <c r="H196" s="11" t="inlineStr">
         <is>
-          <t>Magnolia Oreolu</t>
+          <t>Magnolia Muzlu</t>
         </is>
       </c>
     </row>
@@ -6550,11 +6548,11 @@
       </c>
       <c r="C197" s="11" t="inlineStr">
         <is>
-          <t>Dubai Magnolia</t>
+          <t>Magnolia Oreolu</t>
         </is>
       </c>
       <c r="D197" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E197" s="5" t="n"/>
       <c r="F197" s="5" t="n"/>
@@ -6565,7 +6563,7 @@
       </c>
       <c r="H197" s="11" t="inlineStr">
         <is>
-          <t>Dubai Magnolia</t>
+          <t>Magnolia Oreolu</t>
         </is>
       </c>
     </row>
@@ -6582,18 +6580,22 @@
       </c>
       <c r="C198" s="11" t="inlineStr">
         <is>
-          <t>Supangle</t>
+          <t>Dubai Magnolia</t>
         </is>
       </c>
       <c r="D198" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E198" s="5" t="n"/>
       <c r="F198" s="5" t="n"/>
-      <c r="G198" s="9" t="n"/>
+      <c r="G198" s="9" t="inlineStr">
+        <is>
+          <t>Magnolia</t>
+        </is>
+      </c>
       <c r="H198" s="11" t="inlineStr">
         <is>
-          <t>Supangle</t>
+          <t>Dubai Magnolia</t>
         </is>
       </c>
     </row>
@@ -6610,18 +6612,18 @@
       </c>
       <c r="C199" s="11" t="inlineStr">
         <is>
-          <t>Profiterol Kase</t>
+          <t>Supangle</t>
         </is>
       </c>
       <c r="D199" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E199" s="5" t="n"/>
       <c r="F199" s="5" t="n"/>
       <c r="G199" s="9" t="n"/>
       <c r="H199" s="11" t="inlineStr">
         <is>
-          <t>Profiterol Kase</t>
+          <t>Supangle</t>
         </is>
       </c>
     </row>
@@ -6638,18 +6640,18 @@
       </c>
       <c r="C200" s="11" t="inlineStr">
         <is>
-          <t>Mozaik</t>
+          <t>Profiterol Kase</t>
         </is>
       </c>
       <c r="D200" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E200" s="5" t="n"/>
       <c r="F200" s="5" t="n"/>
       <c r="G200" s="9" t="n"/>
       <c r="H200" s="11" t="inlineStr">
         <is>
-          <t>Mozaik</t>
+          <t>Profiterol Kase</t>
         </is>
       </c>
     </row>
@@ -6666,18 +6668,18 @@
       </c>
       <c r="C201" s="11" t="inlineStr">
         <is>
-          <t>Hasbahçe Tek</t>
+          <t>Mozaik</t>
         </is>
       </c>
       <c r="D201" s="4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E201" s="5" t="n"/>
       <c r="F201" s="5" t="n"/>
       <c r="G201" s="9" t="n"/>
       <c r="H201" s="11" t="inlineStr">
         <is>
-          <t>Hasbahçe Tek</t>
+          <t>Mozaik</t>
         </is>
       </c>
     </row>
@@ -6694,18 +6696,18 @@
       </c>
       <c r="C202" s="11" t="inlineStr">
         <is>
-          <t>Fıstıklı Çikolatalı Tek</t>
+          <t>Hasbahçe Tek</t>
         </is>
       </c>
       <c r="D202" s="4" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E202" s="5" t="n"/>
       <c r="F202" s="5" t="n"/>
       <c r="G202" s="9" t="n"/>
       <c r="H202" s="11" t="inlineStr">
         <is>
-          <t>Fıstıklı Çikolatalı Tek</t>
+          <t>Hasbahçe Tek</t>
         </is>
       </c>
     </row>
@@ -6722,18 +6724,18 @@
       </c>
       <c r="C203" s="11" t="inlineStr">
         <is>
-          <t>Kestaneli Tek</t>
+          <t>Fıstıklı Çikolatalı Tek</t>
         </is>
       </c>
       <c r="D203" s="4" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E203" s="5" t="n"/>
       <c r="F203" s="5" t="n"/>
       <c r="G203" s="9" t="n"/>
       <c r="H203" s="11" t="inlineStr">
         <is>
-          <t>Kestaneli Tek</t>
+          <t>Fıstıklı Çikolatalı Tek</t>
         </is>
       </c>
     </row>
@@ -6750,18 +6752,18 @@
       </c>
       <c r="C204" s="11" t="inlineStr">
         <is>
-          <t>Ganaj Tek</t>
+          <t>Kestaneli Tek</t>
         </is>
       </c>
       <c r="D204" s="4" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E204" s="5" t="n"/>
       <c r="F204" s="5" t="n"/>
       <c r="G204" s="9" t="n"/>
       <c r="H204" s="11" t="inlineStr">
         <is>
-          <t>Ganaj Tek</t>
+          <t>Kestaneli Tek</t>
         </is>
       </c>
     </row>
@@ -6778,71 +6780,67 @@
       </c>
       <c r="C205" s="11" t="inlineStr">
         <is>
-          <t>Latte (Porsiyon)</t>
+          <t>Ganaj Tek</t>
         </is>
       </c>
       <c r="D205" s="4" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E205" s="5" t="n"/>
       <c r="F205" s="5" t="n"/>
       <c r="G205" s="9" t="n"/>
       <c r="H205" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Latte </t>
+          <t>Ganaj Tek</t>
         </is>
       </c>
     </row>
     <row r="206">
-      <c r="A206" s="8" t="inlineStr">
+      <c r="A206" s="11" t="inlineStr">
         <is>
           <t>Porsiyon Tatlılar</t>
         </is>
       </c>
-      <c r="B206" s="8" t="inlineStr">
-        <is>
-          <t>Minik Tatlılar</t>
+      <c r="B206" s="11" t="inlineStr">
+        <is>
+          <t>Porsiyon Tatlılar</t>
         </is>
       </c>
       <c r="C206" s="11" t="inlineStr">
         <is>
-          <t>Çikolatalı Ekler (Porsiyon)</t>
+          <t>Latte (Porsiyon)</t>
         </is>
       </c>
       <c r="D206" s="4" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="E206" s="5" t="n"/>
       <c r="F206" s="5" t="n"/>
-      <c r="G206" s="9" t="inlineStr">
-        <is>
-          <t>Ekler</t>
-        </is>
-      </c>
+      <c r="G206" s="9" t="n"/>
       <c r="H206" s="11" t="inlineStr">
         <is>
-          <t>Çikolatalı Ekler (kg)</t>
+          <t xml:space="preserve">Latte </t>
         </is>
       </c>
     </row>
     <row r="207">
-      <c r="A207" s="11" t="inlineStr">
+      <c r="A207" s="8" t="inlineStr">
         <is>
           <t>Porsiyon Tatlılar</t>
         </is>
       </c>
-      <c r="B207" s="11" t="inlineStr">
+      <c r="B207" s="8" t="inlineStr">
         <is>
           <t>Minik Tatlılar</t>
         </is>
       </c>
       <c r="C207" s="11" t="inlineStr">
         <is>
-          <t>Limonlu Ekler (Porsiyon)</t>
+          <t>Çikolatalı Ekler (Porsiyon)</t>
         </is>
       </c>
       <c r="D207" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E207" s="5" t="n"/>
       <c r="F207" s="5" t="n"/>
@@ -6853,7 +6851,7 @@
       </c>
       <c r="H207" s="11" t="inlineStr">
         <is>
-          <t>Limonlu Ekler (kg)</t>
+          <t>Çikolatalı Ekler (kg)</t>
         </is>
       </c>
     </row>
@@ -6870,11 +6868,11 @@
       </c>
       <c r="C208" s="11" t="inlineStr">
         <is>
-          <t>Beyaz Ekler</t>
+          <t>Limonlu Ekler (Porsiyon)</t>
         </is>
       </c>
       <c r="D208" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E208" s="5" t="n"/>
       <c r="F208" s="5" t="n"/>
@@ -6885,7 +6883,7 @@
       </c>
       <c r="H208" s="11" t="inlineStr">
         <is>
-          <t>Beyaz Ekler (kg)</t>
+          <t>Limonlu Ekler (kg)</t>
         </is>
       </c>
     </row>
@@ -6902,22 +6900,22 @@
       </c>
       <c r="C209" s="11" t="inlineStr">
         <is>
-          <t>Petifür</t>
+          <t>Beyaz Ekler</t>
         </is>
       </c>
       <c r="D209" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E209" s="5" t="n"/>
       <c r="F209" s="5" t="n"/>
       <c r="G209" s="9" t="inlineStr">
         <is>
-          <t>Petifür &amp; Rulo</t>
+          <t>Ekler</t>
         </is>
       </c>
       <c r="H209" s="11" t="inlineStr">
         <is>
-          <t>Petifür (kg)</t>
+          <t>Beyaz Ekler (kg)</t>
         </is>
       </c>
     </row>
@@ -6934,11 +6932,11 @@
       </c>
       <c r="C210" s="11" t="inlineStr">
         <is>
-          <t>Rulo Petifür Muzlu</t>
+          <t>Petifür</t>
         </is>
       </c>
       <c r="D210" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E210" s="5" t="n"/>
       <c r="F210" s="5" t="n"/>
@@ -6949,7 +6947,7 @@
       </c>
       <c r="H210" s="11" t="inlineStr">
         <is>
-          <t>Rulo Petifür Muzlu (kg)</t>
+          <t>Petifür (kg)</t>
         </is>
       </c>
     </row>
@@ -6966,11 +6964,11 @@
       </c>
       <c r="C211" s="11" t="inlineStr">
         <is>
-          <t>Rulo Petifür Çilek</t>
+          <t>Rulo Petifür Muzlu</t>
         </is>
       </c>
       <c r="D211" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E211" s="5" t="n"/>
       <c r="F211" s="5" t="n"/>
@@ -6981,7 +6979,7 @@
       </c>
       <c r="H211" s="11" t="inlineStr">
         <is>
-          <t>Rulo Petifür Çilek (kg)</t>
+          <t>Rulo Petifür Muzlu (kg)</t>
         </is>
       </c>
     </row>
@@ -6998,18 +6996,22 @@
       </c>
       <c r="C212" s="11" t="inlineStr">
         <is>
-          <t>Çiko Limon Parfe</t>
+          <t>Rulo Petifür Çilek</t>
         </is>
       </c>
       <c r="D212" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E212" s="5" t="n"/>
       <c r="F212" s="5" t="n"/>
-      <c r="G212" s="9" t="n"/>
+      <c r="G212" s="9" t="inlineStr">
+        <is>
+          <t>Petifür &amp; Rulo</t>
+        </is>
+      </c>
       <c r="H212" s="11" t="inlineStr">
         <is>
-          <t>Çiko Limon Parfe (kg)</t>
+          <t>Rulo Petifür Çilek (kg)</t>
         </is>
       </c>
     </row>
@@ -7026,22 +7028,18 @@
       </c>
       <c r="C213" s="11" t="inlineStr">
         <is>
-          <t>Çilekli Adet Rulo</t>
+          <t>Çiko Limon Parfe</t>
         </is>
       </c>
       <c r="D213" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E213" s="5" t="n"/>
       <c r="F213" s="5" t="n"/>
-      <c r="G213" s="9" t="inlineStr">
-        <is>
-          <t>Petifür &amp; Rulo</t>
-        </is>
-      </c>
+      <c r="G213" s="9" t="n"/>
       <c r="H213" s="11" t="inlineStr">
         <is>
-          <t>Çilekli Adet Rulo</t>
+          <t>Çiko Limon Parfe (kg)</t>
         </is>
       </c>
     </row>
@@ -7058,11 +7056,11 @@
       </c>
       <c r="C214" s="11" t="inlineStr">
         <is>
-          <t>Muzlu Adet Rulo</t>
+          <t>Çilekli Adet Rulo</t>
         </is>
       </c>
       <c r="D214" s="4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E214" s="5" t="n"/>
       <c r="F214" s="5" t="n"/>
@@ -7073,7 +7071,7 @@
       </c>
       <c r="H214" s="11" t="inlineStr">
         <is>
-          <t>Muzlu Adet Rulo</t>
+          <t>Çilekli Adet Rulo</t>
         </is>
       </c>
     </row>
@@ -7090,22 +7088,22 @@
       </c>
       <c r="C215" s="11" t="inlineStr">
         <is>
-          <t>Krokanlı Şu Topu</t>
+          <t>Muzlu Adet Rulo</t>
         </is>
       </c>
       <c r="D215" s="4" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E215" s="5" t="n"/>
       <c r="F215" s="5" t="n"/>
       <c r="G215" s="9" t="inlineStr">
         <is>
-          <t>Şu Topu</t>
+          <t>Petifür &amp; Rulo</t>
         </is>
       </c>
       <c r="H215" s="11" t="inlineStr">
         <is>
-          <t>Krokanlı Şu Topu</t>
+          <t>Muzlu Adet Rulo</t>
         </is>
       </c>
     </row>
@@ -7122,11 +7120,11 @@
       </c>
       <c r="C216" s="11" t="inlineStr">
         <is>
-          <t>Çilekli Şu Topu</t>
+          <t>Krokanlı Şu Topu</t>
         </is>
       </c>
       <c r="D216" s="4" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E216" s="5" t="n"/>
       <c r="F216" s="5" t="n"/>
@@ -7137,63 +7135,67 @@
       </c>
       <c r="H216" s="11" t="inlineStr">
         <is>
+          <t>Krokanlı Şu Topu</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" s="11" t="inlineStr">
+        <is>
+          <t>Porsiyon Tatlılar</t>
+        </is>
+      </c>
+      <c r="B217" s="11" t="inlineStr">
+        <is>
+          <t>Minik Tatlılar</t>
+        </is>
+      </c>
+      <c r="C217" s="11" t="inlineStr">
+        <is>
           <t>Çilekli Şu Topu</t>
         </is>
       </c>
-    </row>
-    <row r="217">
-      <c r="A217" s="2" t="inlineStr">
-        <is>
-          <t>Porsiyon Tatlılar</t>
-        </is>
-      </c>
-      <c r="B217" s="2" t="inlineStr">
-        <is>
-          <t>Sütlü Tatlı</t>
-        </is>
-      </c>
-      <c r="C217" s="11" t="inlineStr">
-        <is>
-          <t>Kazandibi</t>
-        </is>
-      </c>
       <c r="D217" s="4" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="E217" s="5" t="n"/>
       <c r="F217" s="5" t="n"/>
-      <c r="G217" s="9" t="n"/>
+      <c r="G217" s="9" t="inlineStr">
+        <is>
+          <t>Şu Topu</t>
+        </is>
+      </c>
       <c r="H217" s="11" t="inlineStr">
         <is>
+          <t>Çilekli Şu Topu</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" s="2" t="inlineStr">
+        <is>
+          <t>Porsiyon Tatlılar</t>
+        </is>
+      </c>
+      <c r="B218" s="2" t="inlineStr">
+        <is>
+          <t>Sütlü Tatlı</t>
+        </is>
+      </c>
+      <c r="C218" s="11" t="inlineStr">
+        <is>
           <t>Kazandibi</t>
         </is>
       </c>
-    </row>
-    <row r="218">
-      <c r="A218" s="11" t="inlineStr">
-        <is>
-          <t>Porsiyon Tatlılar</t>
-        </is>
-      </c>
-      <c r="B218" s="11" t="inlineStr">
-        <is>
-          <t>Sütlü Tatlı</t>
-        </is>
-      </c>
-      <c r="C218" s="11" t="inlineStr">
-        <is>
-          <t>Sütlaç</t>
-        </is>
-      </c>
       <c r="D218" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E218" s="5" t="n"/>
       <c r="F218" s="5" t="n"/>
       <c r="G218" s="9" t="n"/>
       <c r="H218" s="11" t="inlineStr">
         <is>
-          <t>Sütlaç</t>
+          <t>Kazandibi</t>
         </is>
       </c>
     </row>
@@ -7210,18 +7212,18 @@
       </c>
       <c r="C219" s="11" t="inlineStr">
         <is>
-          <t>Aşure</t>
+          <t>Sütlaç</t>
         </is>
       </c>
       <c r="D219" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E219" s="5" t="n"/>
       <c r="F219" s="5" t="n"/>
       <c r="G219" s="9" t="n"/>
       <c r="H219" s="11" t="inlineStr">
         <is>
-          <t>Aşure</t>
+          <t>Sütlaç</t>
         </is>
       </c>
     </row>
@@ -7233,27 +7235,23 @@
       </c>
       <c r="B220" s="11" t="inlineStr">
         <is>
-          <t>Porsiyon Tatlılar</t>
+          <t>Sütlü Tatlı</t>
         </is>
       </c>
       <c r="C220" s="11" t="inlineStr">
         <is>
-          <t>Trileçe Frambuaz</t>
+          <t>Aşure</t>
         </is>
       </c>
       <c r="D220" s="4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E220" s="5" t="n"/>
       <c r="F220" s="5" t="n"/>
-      <c r="G220" s="9" t="inlineStr">
-        <is>
-          <t>Trileçe</t>
-        </is>
-      </c>
+      <c r="G220" s="9" t="n"/>
       <c r="H220" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Frambuaz Triliçe</t>
+          <t>Aşure</t>
         </is>
       </c>
     </row>
@@ -7270,11 +7268,11 @@
       </c>
       <c r="C221" s="11" t="inlineStr">
         <is>
-          <t>Trileçe Karamel</t>
+          <t>Trileçe Frambuaz</t>
         </is>
       </c>
       <c r="D221" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E221" s="5" t="n"/>
       <c r="F221" s="5" t="n"/>
@@ -7284,6 +7282,38 @@
         </is>
       </c>
       <c r="H221" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Frambuaz Triliçe</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="11" t="inlineStr">
+        <is>
+          <t>Porsiyon Tatlılar</t>
+        </is>
+      </c>
+      <c r="B222" s="11" t="inlineStr">
+        <is>
+          <t>Porsiyon Tatlılar</t>
+        </is>
+      </c>
+      <c r="C222" s="11" t="inlineStr">
+        <is>
+          <t>Trileçe Karamel</t>
+        </is>
+      </c>
+      <c r="D222" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E222" s="5" t="n"/>
+      <c r="F222" s="5" t="n"/>
+      <c r="G222" s="9" t="inlineStr">
+        <is>
+          <t>Trileçe</t>
+        </is>
+      </c>
+      <c r="H222" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve"> Karamel Triliçe</t>
         </is>

</xml_diff>

<commit_message>
Sebzeli'yi Cevizli Kekikli Sarma'nın altına taşı
</commit_message>
<xml_diff>
--- a/rapor-duzeni.xlsx
+++ b/rapor-duzeni.xlsx
@@ -4960,34 +4960,32 @@
       </c>
     </row>
     <row r="148">
-      <c r="A148" s="11" t="inlineStr">
+      <c r="A148" t="inlineStr">
         <is>
           <t>Tuzlu Kurabiye</t>
         </is>
       </c>
-      <c r="B148" s="11" t="inlineStr">
+      <c r="B148" t="inlineStr">
         <is>
           <t>Börekli Taş &amp; Poğaça Grubu</t>
         </is>
       </c>
-      <c r="C148" s="11" t="inlineStr">
-        <is>
-          <t>Kornet Dereotlu</t>
-        </is>
-      </c>
-      <c r="D148" s="4" t="n">
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>Sebzeli</t>
+        </is>
+      </c>
+      <c r="D148" t="n">
         <v>7</v>
       </c>
-      <c r="E148" s="5" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="F148" s="5" t="n"/>
-      <c r="G148" s="9" t="n"/>
-      <c r="H148" s="11" t="inlineStr">
-        <is>
-          <t>Kornet Dereotlu</t>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>tp</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>Sebzeli</t>
         </is>
       </c>
     </row>
@@ -5004,7 +5002,7 @@
       </c>
       <c r="C149" s="11" t="inlineStr">
         <is>
-          <t>Dereotlu Sufle</t>
+          <t>Kornet Dereotlu</t>
         </is>
       </c>
       <c r="D149" s="4" t="n">
@@ -5019,7 +5017,7 @@
       <c r="G149" s="9" t="n"/>
       <c r="H149" s="11" t="inlineStr">
         <is>
-          <t>Dereotlu Sufle</t>
+          <t>Kornet Dereotlu</t>
         </is>
       </c>
     </row>
@@ -5036,7 +5034,7 @@
       </c>
       <c r="C150" s="11" t="inlineStr">
         <is>
-          <t>Sebzeli</t>
+          <t>Dereotlu Sufle</t>
         </is>
       </c>
       <c r="D150" s="4" t="n">
@@ -5044,14 +5042,14 @@
       </c>
       <c r="E150" s="5" t="inlineStr">
         <is>
-          <t>tp</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="F150" s="5" t="n"/>
       <c r="G150" s="9" t="n"/>
       <c r="H150" s="11" t="inlineStr">
         <is>
-          <t>Sebzeli</t>
+          <t>Dereotlu Sufle</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Patlıcanlı ürününü listeden çıkar
</commit_message>
<xml_diff>
--- a/rapor-duzeni.xlsx
+++ b/rapor-duzeni.xlsx
@@ -500,7 +500,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H222"/>
+  <dimension ref="A1:H221"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5066,7 +5066,7 @@
       </c>
       <c r="C151" s="11" t="inlineStr">
         <is>
-          <t>Patlıcanlı</t>
+          <t>Mini Pizza</t>
         </is>
       </c>
       <c r="D151" s="4" t="n">
@@ -5081,7 +5081,7 @@
       <c r="G151" s="9" t="n"/>
       <c r="H151" s="11" t="inlineStr">
         <is>
-          <t>Patlıcanlı</t>
+          <t>Mini Pizza</t>
         </is>
       </c>
     </row>
@@ -5098,7 +5098,7 @@
       </c>
       <c r="C152" s="11" t="inlineStr">
         <is>
-          <t>Mini Pizza</t>
+          <t>Minik Simit</t>
         </is>
       </c>
       <c r="D152" s="4" t="n">
@@ -5113,7 +5113,7 @@
       <c r="G152" s="9" t="n"/>
       <c r="H152" s="11" t="inlineStr">
         <is>
-          <t>Mini Pizza</t>
+          <t>Minik Simit</t>
         </is>
       </c>
     </row>
@@ -5130,7 +5130,7 @@
       </c>
       <c r="C153" s="11" t="inlineStr">
         <is>
-          <t>Minik Simit</t>
+          <t>Düz Örgü</t>
         </is>
       </c>
       <c r="D153" s="4" t="n">
@@ -5145,7 +5145,7 @@
       <c r="G153" s="9" t="n"/>
       <c r="H153" s="11" t="inlineStr">
         <is>
-          <t>Minik Simit</t>
+          <t>Düz Örgü</t>
         </is>
       </c>
     </row>
@@ -5162,7 +5162,7 @@
       </c>
       <c r="C154" s="11" t="inlineStr">
         <is>
-          <t>Düz Örgü</t>
+          <t>Yuvarlak Örgü</t>
         </is>
       </c>
       <c r="D154" s="4" t="n">
@@ -5177,7 +5177,7 @@
       <c r="G154" s="9" t="n"/>
       <c r="H154" s="11" t="inlineStr">
         <is>
-          <t>Düz Örgü</t>
+          <t>Yuvarlak Örgü</t>
         </is>
       </c>
     </row>
@@ -5194,7 +5194,7 @@
       </c>
       <c r="C155" s="11" t="inlineStr">
         <is>
-          <t>Yuvarlak Örgü</t>
+          <t>Burgu Susamlı Haşhaşlı</t>
         </is>
       </c>
       <c r="D155" s="4" t="n">
@@ -5209,67 +5209,67 @@
       <c r="G155" s="9" t="n"/>
       <c r="H155" s="11" t="inlineStr">
         <is>
-          <t>Yuvarlak Örgü</t>
+          <t>Burgu Susamlı Haşhaşlı</t>
         </is>
       </c>
     </row>
     <row r="156">
-      <c r="A156" s="11" t="inlineStr">
+      <c r="A156" s="2" t="inlineStr">
         <is>
           <t>Tuzlu Kurabiye</t>
         </is>
       </c>
-      <c r="B156" s="11" t="inlineStr">
-        <is>
-          <t>Börekli Taş &amp; Poğaça Grubu</t>
+      <c r="B156" s="2" t="inlineStr">
+        <is>
+          <t>Diyet Kurabiyeler</t>
         </is>
       </c>
       <c r="C156" s="11" t="inlineStr">
         <is>
-          <t>Burgu Susamlı Haşhaşlı</t>
+          <t>Burgu Tahıllı</t>
         </is>
       </c>
       <c r="D156" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="E156" s="5" t="inlineStr">
-        <is>
-          <t>tp</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="E156" s="5" t="n"/>
       <c r="F156" s="5" t="n"/>
       <c r="G156" s="9" t="n"/>
       <c r="H156" s="11" t="inlineStr">
         <is>
-          <t>Burgu Susamlı Haşhaşlı</t>
+          <t>Burgu Tahıllı</t>
         </is>
       </c>
     </row>
     <row r="157">
-      <c r="A157" s="2" t="inlineStr">
+      <c r="A157" s="11" t="inlineStr">
         <is>
           <t>Tuzlu Kurabiye</t>
         </is>
       </c>
-      <c r="B157" s="2" t="inlineStr">
+      <c r="B157" s="11" t="inlineStr">
         <is>
           <t>Diyet Kurabiyeler</t>
         </is>
       </c>
       <c r="C157" s="11" t="inlineStr">
         <is>
-          <t>Burgu Tahıllı</t>
+          <t>Ayçekirdekli Galeta</t>
         </is>
       </c>
       <c r="D157" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E157" s="5" t="n"/>
+        <v>2</v>
+      </c>
+      <c r="E157" s="5" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
       <c r="F157" s="5" t="n"/>
       <c r="G157" s="9" t="n"/>
       <c r="H157" s="11" t="inlineStr">
         <is>
-          <t>Burgu Tahıllı</t>
+          <t>Ayçekirdekli Galeta</t>
         </is>
       </c>
     </row>
@@ -5286,22 +5286,22 @@
       </c>
       <c r="C158" s="11" t="inlineStr">
         <is>
-          <t>Ayçekirdekli Galeta</t>
+          <t>Parmesan Galeta</t>
         </is>
       </c>
       <c r="D158" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E158" s="5" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>tp</t>
         </is>
       </c>
       <c r="F158" s="5" t="n"/>
       <c r="G158" s="9" t="n"/>
       <c r="H158" s="11" t="inlineStr">
         <is>
-          <t>Ayçekirdekli Galeta</t>
+          <t>Parmesan Galeta</t>
         </is>
       </c>
     </row>
@@ -5318,11 +5318,11 @@
       </c>
       <c r="C159" s="11" t="inlineStr">
         <is>
-          <t>Parmesan Galeta</t>
+          <t>İtalyan Galeta</t>
         </is>
       </c>
       <c r="D159" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E159" s="5" t="inlineStr">
         <is>
@@ -5333,7 +5333,7 @@
       <c r="G159" s="9" t="n"/>
       <c r="H159" s="11" t="inlineStr">
         <is>
-          <t>Parmesan Galeta</t>
+          <t>İtalyan Galeta</t>
         </is>
       </c>
     </row>
@@ -5350,11 +5350,11 @@
       </c>
       <c r="C160" s="11" t="inlineStr">
         <is>
-          <t>İtalyan Galeta</t>
+          <t>Biberiyeli Zeytinli Galeta</t>
         </is>
       </c>
       <c r="D160" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E160" s="5" t="inlineStr">
         <is>
@@ -5365,7 +5365,7 @@
       <c r="G160" s="9" t="n"/>
       <c r="H160" s="11" t="inlineStr">
         <is>
-          <t>İtalyan Galeta</t>
+          <t>Biberiyeli Zeytinli Galeta</t>
         </is>
       </c>
     </row>
@@ -5382,11 +5382,11 @@
       </c>
       <c r="C161" s="11" t="inlineStr">
         <is>
-          <t>Biberiyeli Zeytinli Galeta</t>
+          <t>Çekirdekli Kokteyl</t>
         </is>
       </c>
       <c r="D161" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E161" s="5" t="inlineStr">
         <is>
@@ -5397,7 +5397,7 @@
       <c r="G161" s="9" t="n"/>
       <c r="H161" s="11" t="inlineStr">
         <is>
-          <t>Biberiyeli Zeytinli Galeta</t>
+          <t>Çekirdekli Kokteyl</t>
         </is>
       </c>
     </row>
@@ -5414,11 +5414,11 @@
       </c>
       <c r="C162" s="11" t="inlineStr">
         <is>
-          <t>Çekirdekli Kokteyl</t>
+          <t>Üzümlü Kepekli</t>
         </is>
       </c>
       <c r="D162" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E162" s="5" t="inlineStr">
         <is>
@@ -5429,7 +5429,7 @@
       <c r="G162" s="9" t="n"/>
       <c r="H162" s="11" t="inlineStr">
         <is>
-          <t>Çekirdekli Kokteyl</t>
+          <t>Üzümlü Kepekli</t>
         </is>
       </c>
     </row>
@@ -5446,11 +5446,11 @@
       </c>
       <c r="C163" s="11" t="inlineStr">
         <is>
-          <t>Üzümlü Kepekli</t>
+          <t>Üzümlü Cevizli Kepekli</t>
         </is>
       </c>
       <c r="D163" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E163" s="5" t="inlineStr">
         <is>
@@ -5461,7 +5461,7 @@
       <c r="G163" s="9" t="n"/>
       <c r="H163" s="11" t="inlineStr">
         <is>
-          <t>Üzümlü Kepekli</t>
+          <t>Üzümlü Cevizli Kepekli</t>
         </is>
       </c>
     </row>
@@ -5478,22 +5478,18 @@
       </c>
       <c r="C164" s="11" t="inlineStr">
         <is>
-          <t>Üzümlü Cevizli Kepekli</t>
+          <t>Kuru Üzümlü Yassı Tahıllı</t>
         </is>
       </c>
       <c r="D164" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="E164" s="5" t="inlineStr">
-        <is>
-          <t>tp</t>
-        </is>
-      </c>
+        <v>9</v>
+      </c>
+      <c r="E164" s="5" t="n"/>
       <c r="F164" s="5" t="n"/>
       <c r="G164" s="9" t="n"/>
       <c r="H164" s="11" t="inlineStr">
         <is>
-          <t>Üzümlü Cevizli Kepekli</t>
+          <t>Kuru Üzümlü Yassı Tahıllı</t>
         </is>
       </c>
     </row>
@@ -5510,18 +5506,22 @@
       </c>
       <c r="C165" s="11" t="inlineStr">
         <is>
-          <t>Kuru Üzümlü Yassı Tahıllı</t>
+          <t>Granola Bar Tepsi</t>
         </is>
       </c>
       <c r="D165" s="4" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E165" s="5" t="n"/>
       <c r="F165" s="5" t="n"/>
-      <c r="G165" s="9" t="n"/>
+      <c r="G165" s="9" t="inlineStr">
+        <is>
+          <t>Bar</t>
+        </is>
+      </c>
       <c r="H165" s="11" t="inlineStr">
         <is>
-          <t>Kuru Üzümlü Yassı Tahıllı</t>
+          <t>Granola Bar Tepsi</t>
         </is>
       </c>
     </row>
@@ -5538,22 +5538,18 @@
       </c>
       <c r="C166" s="11" t="inlineStr">
         <is>
-          <t>Granola Bar Tepsi</t>
+          <t>Tahinli Susamlı</t>
         </is>
       </c>
       <c r="D166" s="4" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E166" s="5" t="n"/>
       <c r="F166" s="5" t="n"/>
-      <c r="G166" s="9" t="inlineStr">
-        <is>
-          <t>Bar</t>
-        </is>
-      </c>
+      <c r="G166" s="9" t="n"/>
       <c r="H166" s="11" t="inlineStr">
         <is>
-          <t>Granola Bar Tepsi</t>
+          <t>Tahinli Susamlı</t>
         </is>
       </c>
     </row>
@@ -5570,18 +5566,18 @@
       </c>
       <c r="C167" s="11" t="inlineStr">
         <is>
-          <t>Tahinli Susamlı</t>
+          <t>Granola Dökme</t>
         </is>
       </c>
       <c r="D167" s="4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E167" s="5" t="n"/>
       <c r="F167" s="5" t="n"/>
       <c r="G167" s="9" t="n"/>
       <c r="H167" s="11" t="inlineStr">
         <is>
-          <t>Tahinli Susamlı</t>
+          <t>Granola Dökme</t>
         </is>
       </c>
     </row>
@@ -5598,74 +5594,74 @@
       </c>
       <c r="C168" s="11" t="inlineStr">
         <is>
-          <t>Granola Dökme</t>
+          <t>Kalp Denge Tahıllı</t>
         </is>
       </c>
       <c r="D168" s="4" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E168" s="5" t="n"/>
       <c r="F168" s="5" t="n"/>
       <c r="G168" s="9" t="n"/>
       <c r="H168" s="11" t="inlineStr">
         <is>
-          <t>Granola Dökme</t>
+          <t>Kalp Denge Tahıllı</t>
         </is>
       </c>
     </row>
     <row r="169">
-      <c r="A169" s="11" t="inlineStr">
+      <c r="A169" s="2" t="inlineStr">
         <is>
           <t>Tuzlu Kurabiye</t>
         </is>
       </c>
-      <c r="B169" s="11" t="inlineStr">
-        <is>
-          <t>Diyet Kurabiyeler</t>
+      <c r="B169" s="2" t="inlineStr">
+        <is>
+          <t>Adet Ürünler</t>
         </is>
       </c>
       <c r="C169" s="11" t="inlineStr">
         <is>
-          <t>Kalp Denge Tahıllı</t>
+          <t>Paskalya</t>
         </is>
       </c>
       <c r="D169" s="4" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="E169" s="5" t="n"/>
       <c r="F169" s="5" t="n"/>
       <c r="G169" s="9" t="n"/>
       <c r="H169" s="11" t="inlineStr">
         <is>
-          <t>Kalp Denge Tahıllı</t>
+          <t>Paskalya</t>
         </is>
       </c>
     </row>
     <row r="170">
-      <c r="A170" s="2" t="inlineStr">
+      <c r="A170" s="11" t="inlineStr">
         <is>
           <t>Tuzlu Kurabiye</t>
         </is>
       </c>
-      <c r="B170" s="2" t="inlineStr">
+      <c r="B170" s="11" t="inlineStr">
         <is>
           <t>Adet Ürünler</t>
         </is>
       </c>
       <c r="C170" s="11" t="inlineStr">
         <is>
-          <t>Paskalya</t>
+          <t>Paskalya Çikolatalı</t>
         </is>
       </c>
       <c r="D170" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E170" s="5" t="n"/>
       <c r="F170" s="5" t="n"/>
       <c r="G170" s="9" t="n"/>
       <c r="H170" s="11" t="inlineStr">
         <is>
-          <t>Paskalya</t>
+          <t>Paskalya Çikolatalı</t>
         </is>
       </c>
     </row>
@@ -5682,18 +5678,18 @@
       </c>
       <c r="C171" s="11" t="inlineStr">
         <is>
-          <t>Paskalya Çikolatalı</t>
+          <t>Tahinli Çörek</t>
         </is>
       </c>
       <c r="D171" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E171" s="5" t="n"/>
       <c r="F171" s="5" t="n"/>
       <c r="G171" s="9" t="n"/>
       <c r="H171" s="11" t="inlineStr">
         <is>
-          <t>Paskalya Çikolatalı</t>
+          <t>Tahinli Çörek</t>
         </is>
       </c>
     </row>
@@ -5710,18 +5706,22 @@
       </c>
       <c r="C172" s="11" t="inlineStr">
         <is>
-          <t>Tahinli Çörek</t>
+          <t>Beze Büyük</t>
         </is>
       </c>
       <c r="D172" s="4" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E172" s="5" t="n"/>
       <c r="F172" s="5" t="n"/>
-      <c r="G172" s="9" t="n"/>
+      <c r="G172" s="9" t="inlineStr">
+        <is>
+          <t>Beze</t>
+        </is>
+      </c>
       <c r="H172" s="11" t="inlineStr">
         <is>
-          <t>Tahinli Çörek</t>
+          <t>Beze Büyük</t>
         </is>
       </c>
     </row>
@@ -5738,11 +5738,11 @@
       </c>
       <c r="C173" s="11" t="inlineStr">
         <is>
-          <t>Beze Büyük</t>
+          <t>Beze Beyaz Minik</t>
         </is>
       </c>
       <c r="D173" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E173" s="5" t="n"/>
       <c r="F173" s="5" t="n"/>
@@ -5753,7 +5753,7 @@
       </c>
       <c r="H173" s="11" t="inlineStr">
         <is>
-          <t>Beze Büyük</t>
+          <t>Beze Beyaz Minik</t>
         </is>
       </c>
     </row>
@@ -5770,11 +5770,11 @@
       </c>
       <c r="C174" s="11" t="inlineStr">
         <is>
-          <t>Beze Beyaz Minik</t>
+          <t>Beze Renkli Minik</t>
         </is>
       </c>
       <c r="D174" s="4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E174" s="5" t="n"/>
       <c r="F174" s="5" t="n"/>
@@ -5785,7 +5785,7 @@
       </c>
       <c r="H174" s="11" t="inlineStr">
         <is>
-          <t>Beze Beyaz Minik</t>
+          <t>Beze Renkli Minik</t>
         </is>
       </c>
     </row>
@@ -5802,22 +5802,18 @@
       </c>
       <c r="C175" s="11" t="inlineStr">
         <is>
-          <t>Beze Renkli Minik</t>
+          <t>Acıbadem</t>
         </is>
       </c>
       <c r="D175" s="4" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="E175" s="5" t="n"/>
       <c r="F175" s="5" t="n"/>
-      <c r="G175" s="9" t="inlineStr">
-        <is>
-          <t>Beze</t>
-        </is>
-      </c>
+      <c r="G175" s="9" t="n"/>
       <c r="H175" s="11" t="inlineStr">
         <is>
-          <t>Beze Renkli Minik</t>
+          <t>Acıbadem</t>
         </is>
       </c>
     </row>
@@ -5834,18 +5830,18 @@
       </c>
       <c r="C176" s="11" t="inlineStr">
         <is>
-          <t>Acıbadem</t>
+          <t>Acıbadem Minik</t>
         </is>
       </c>
       <c r="D176" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E176" s="5" t="n"/>
       <c r="F176" s="5" t="n"/>
       <c r="G176" s="9" t="n"/>
       <c r="H176" s="11" t="inlineStr">
         <is>
-          <t>Acıbadem</t>
+          <t>Acıbadem Minik</t>
         </is>
       </c>
     </row>
@@ -5862,67 +5858,75 @@
       </c>
       <c r="C177" s="11" t="inlineStr">
         <is>
-          <t>Acıbadem Minik</t>
+          <t>Ayçöreği</t>
         </is>
       </c>
       <c r="D177" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E177" s="5" t="n"/>
       <c r="F177" s="5" t="n"/>
       <c r="G177" s="9" t="n"/>
       <c r="H177" s="11" t="inlineStr">
         <is>
-          <t>Acıbadem Minik</t>
+          <t>Ayçöreği</t>
         </is>
       </c>
     </row>
     <row r="178">
-      <c r="A178" s="11" t="inlineStr">
+      <c r="A178" s="2" t="inlineStr">
         <is>
           <t>Tuzlu Kurabiye</t>
         </is>
       </c>
-      <c r="B178" s="11" t="inlineStr">
-        <is>
-          <t>Adet Ürünler</t>
+      <c r="B178" s="2" t="inlineStr">
+        <is>
+          <t>Galeta / Kıtır / Cips / Diğer Tuzlu</t>
         </is>
       </c>
       <c r="C178" s="11" t="inlineStr">
         <is>
-          <t>Ayçöreği</t>
+          <t>Batonsale Sade</t>
         </is>
       </c>
       <c r="D178" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="E178" s="5" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="E178" s="5" t="inlineStr">
+        <is>
+          <t>tp</t>
+        </is>
+      </c>
       <c r="F178" s="5" t="n"/>
-      <c r="G178" s="9" t="n"/>
+      <c r="G178" s="9" t="inlineStr">
+        <is>
+          <t>Batonsale</t>
+        </is>
+      </c>
       <c r="H178" s="11" t="inlineStr">
         <is>
-          <t>Ayçöreği</t>
+          <t>Batonsale Sade</t>
         </is>
       </c>
     </row>
     <row r="179">
-      <c r="A179" s="2" t="inlineStr">
+      <c r="A179" s="11" t="inlineStr">
         <is>
           <t>Tuzlu Kurabiye</t>
         </is>
       </c>
-      <c r="B179" s="2" t="inlineStr">
+      <c r="B179" s="11" t="inlineStr">
         <is>
           <t>Galeta / Kıtır / Cips / Diğer Tuzlu</t>
         </is>
       </c>
       <c r="C179" s="11" t="inlineStr">
         <is>
-          <t>Batonsale Sade</t>
+          <t>Batonsale Çörekotlu</t>
         </is>
       </c>
       <c r="D179" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E179" s="5" t="inlineStr">
         <is>
@@ -5937,7 +5941,7 @@
       </c>
       <c r="H179" s="11" t="inlineStr">
         <is>
-          <t>Batonsale Sade</t>
+          <t>Batonsale Çörekotlu</t>
         </is>
       </c>
     </row>
@@ -5954,11 +5958,11 @@
       </c>
       <c r="C180" s="11" t="inlineStr">
         <is>
-          <t>Batonsale Çörekotlu</t>
+          <t>Batonsale Kaşarlı</t>
         </is>
       </c>
       <c r="D180" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E180" s="5" t="inlineStr">
         <is>
@@ -5973,7 +5977,7 @@
       </c>
       <c r="H180" s="11" t="inlineStr">
         <is>
-          <t>Batonsale Çörekotlu</t>
+          <t>Batonsale Kaşarlı</t>
         </is>
       </c>
     </row>
@@ -5990,11 +5994,11 @@
       </c>
       <c r="C181" s="11" t="inlineStr">
         <is>
-          <t>Batonsale Kaşarlı</t>
+          <t>Kırık Kırak Susamlı</t>
         </is>
       </c>
       <c r="D181" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E181" s="5" t="inlineStr">
         <is>
@@ -6002,14 +6006,10 @@
         </is>
       </c>
       <c r="F181" s="5" t="n"/>
-      <c r="G181" s="9" t="inlineStr">
-        <is>
-          <t>Batonsale</t>
-        </is>
-      </c>
+      <c r="G181" s="9" t="n"/>
       <c r="H181" s="11" t="inlineStr">
         <is>
-          <t>Batonsale Kaşarlı</t>
+          <t>Kırık Kırak Susamlı</t>
         </is>
       </c>
     </row>
@@ -6026,11 +6026,11 @@
       </c>
       <c r="C182" s="11" t="inlineStr">
         <is>
-          <t>Kırık Kırak Susamlı</t>
+          <t>Galet Kaşarlı</t>
         </is>
       </c>
       <c r="D182" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E182" s="5" t="inlineStr">
         <is>
@@ -6038,10 +6038,14 @@
         </is>
       </c>
       <c r="F182" s="5" t="n"/>
-      <c r="G182" s="9" t="n"/>
+      <c r="G182" s="9" t="inlineStr">
+        <is>
+          <t>Galet</t>
+        </is>
+      </c>
       <c r="H182" s="11" t="inlineStr">
         <is>
-          <t>Kırık Kırak Susamlı</t>
+          <t>Galet Kaşarlı</t>
         </is>
       </c>
     </row>
@@ -6058,11 +6062,11 @@
       </c>
       <c r="C183" s="11" t="inlineStr">
         <is>
-          <t>Galet Kaşarlı</t>
+          <t>Galet Çörekotlu</t>
         </is>
       </c>
       <c r="D183" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E183" s="5" t="inlineStr">
         <is>
@@ -6077,7 +6081,7 @@
       </c>
       <c r="H183" s="11" t="inlineStr">
         <is>
-          <t>Galet Kaşarlı</t>
+          <t>Galet Çörekotlu</t>
         </is>
       </c>
     </row>
@@ -6094,11 +6098,11 @@
       </c>
       <c r="C184" s="11" t="inlineStr">
         <is>
-          <t>Galet Çörekotlu</t>
+          <t>Galet Susamlı</t>
         </is>
       </c>
       <c r="D184" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E184" s="5" t="inlineStr">
         <is>
@@ -6113,7 +6117,7 @@
       </c>
       <c r="H184" s="11" t="inlineStr">
         <is>
-          <t>Galet Çörekotlu</t>
+          <t>Galet Susamlı</t>
         </is>
       </c>
     </row>
@@ -6130,11 +6134,11 @@
       </c>
       <c r="C185" s="11" t="inlineStr">
         <is>
-          <t>Galet Susamlı</t>
+          <t>Baharatlı Kıtır</t>
         </is>
       </c>
       <c r="D185" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E185" s="5" t="inlineStr">
         <is>
@@ -6144,12 +6148,12 @@
       <c r="F185" s="5" t="n"/>
       <c r="G185" s="9" t="inlineStr">
         <is>
-          <t>Galet</t>
+          <t>Kıtır</t>
         </is>
       </c>
       <c r="H185" s="11" t="inlineStr">
         <is>
-          <t>Galet Susamlı</t>
+          <t>Baharatlı Kıtır</t>
         </is>
       </c>
     </row>
@@ -6166,11 +6170,11 @@
       </c>
       <c r="C186" s="11" t="inlineStr">
         <is>
-          <t>Baharatlı Kıtır</t>
+          <t>Kaşarlı Kıtır</t>
         </is>
       </c>
       <c r="D186" s="4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E186" s="5" t="inlineStr">
         <is>
@@ -6185,7 +6189,7 @@
       </c>
       <c r="H186" s="11" t="inlineStr">
         <is>
-          <t>Baharatlı Kıtır</t>
+          <t>Kaşarlı Kıtır</t>
         </is>
       </c>
     </row>
@@ -6202,11 +6206,11 @@
       </c>
       <c r="C187" s="11" t="inlineStr">
         <is>
-          <t>Kaşarlı Kıtır</t>
+          <t>Zencefilli Kıtır</t>
         </is>
       </c>
       <c r="D187" s="4" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E187" s="5" t="inlineStr">
         <is>
@@ -6221,7 +6225,7 @@
       </c>
       <c r="H187" s="11" t="inlineStr">
         <is>
-          <t>Kaşarlı Kıtır</t>
+          <t>Zencefilli Kıtır</t>
         </is>
       </c>
     </row>
@@ -6238,11 +6242,11 @@
       </c>
       <c r="C188" s="11" t="inlineStr">
         <is>
-          <t>Zencefilli Kıtır</t>
+          <t>Acılı Kıtır</t>
         </is>
       </c>
       <c r="D188" s="4" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E188" s="5" t="inlineStr">
         <is>
@@ -6257,7 +6261,7 @@
       </c>
       <c r="H188" s="11" t="inlineStr">
         <is>
-          <t>Zencefilli Kıtır</t>
+          <t>Acılı Kıtır</t>
         </is>
       </c>
     </row>
@@ -6274,11 +6278,11 @@
       </c>
       <c r="C189" s="11" t="inlineStr">
         <is>
-          <t>Acılı Kıtır</t>
+          <t>Haşhaşlı Cips</t>
         </is>
       </c>
       <c r="D189" s="4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E189" s="5" t="inlineStr">
         <is>
@@ -6288,12 +6292,12 @@
       <c r="F189" s="5" t="n"/>
       <c r="G189" s="9" t="inlineStr">
         <is>
-          <t>Kıtır</t>
+          <t>Cips</t>
         </is>
       </c>
       <c r="H189" s="11" t="inlineStr">
         <is>
-          <t>Acılı Kıtır</t>
+          <t>Haşhaşlı Cips</t>
         </is>
       </c>
     </row>
@@ -6310,11 +6314,11 @@
       </c>
       <c r="C190" s="11" t="inlineStr">
         <is>
-          <t>Haşhaşlı Cips</t>
+          <t>İrmikli Cips</t>
         </is>
       </c>
       <c r="D190" s="4" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E190" s="5" t="inlineStr">
         <is>
@@ -6329,7 +6333,7 @@
       </c>
       <c r="H190" s="11" t="inlineStr">
         <is>
-          <t>Haşhaşlı Cips</t>
+          <t>İrmikli Cips</t>
         </is>
       </c>
     </row>
@@ -6346,11 +6350,11 @@
       </c>
       <c r="C191" s="11" t="inlineStr">
         <is>
-          <t>İrmikli Cips</t>
+          <t>Parmesanlı Cips</t>
         </is>
       </c>
       <c r="D191" s="4" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E191" s="5" t="inlineStr">
         <is>
@@ -6365,7 +6369,7 @@
       </c>
       <c r="H191" s="11" t="inlineStr">
         <is>
-          <t>İrmikli Cips</t>
+          <t>Parmesanlı Cips</t>
         </is>
       </c>
     </row>
@@ -6382,11 +6386,11 @@
       </c>
       <c r="C192" s="11" t="inlineStr">
         <is>
-          <t>Parmesanlı Cips</t>
+          <t>Tam Buğday Cips</t>
         </is>
       </c>
       <c r="D192" s="4" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E192" s="5" t="inlineStr">
         <is>
@@ -6401,71 +6405,67 @@
       </c>
       <c r="H192" s="11" t="inlineStr">
         <is>
-          <t>Parmesanlı Cips</t>
+          <t>Tam Buğday Cips</t>
         </is>
       </c>
     </row>
     <row r="193">
-      <c r="A193" s="11" t="inlineStr">
-        <is>
-          <t>Tuzlu Kurabiye</t>
-        </is>
-      </c>
-      <c r="B193" s="11" t="inlineStr">
-        <is>
-          <t>Galeta / Kıtır / Cips / Diğer Tuzlu</t>
+      <c r="A193" s="2" t="inlineStr">
+        <is>
+          <t>Porsiyon Tatlılar</t>
+        </is>
+      </c>
+      <c r="B193" s="2" t="inlineStr">
+        <is>
+          <t>Porsiyon Tatlılar</t>
         </is>
       </c>
       <c r="C193" s="11" t="inlineStr">
         <is>
-          <t>Tam Buğday Cips</t>
+          <t>Tiramisu Dilim</t>
         </is>
       </c>
       <c r="D193" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="E193" s="5" t="inlineStr">
-        <is>
-          <t>tp</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="E193" s="5" t="n"/>
       <c r="F193" s="5" t="n"/>
-      <c r="G193" s="9" t="inlineStr">
-        <is>
-          <t>Cips</t>
-        </is>
-      </c>
+      <c r="G193" s="9" t="n"/>
       <c r="H193" s="11" t="inlineStr">
         <is>
-          <t>Tam Buğday Cips</t>
+          <t>Tiramisu Dilim</t>
         </is>
       </c>
     </row>
     <row r="194">
-      <c r="A194" s="2" t="inlineStr">
+      <c r="A194" s="11" t="inlineStr">
         <is>
           <t>Porsiyon Tatlılar</t>
         </is>
       </c>
-      <c r="B194" s="2" t="inlineStr">
+      <c r="B194" s="11" t="inlineStr">
         <is>
           <t>Porsiyon Tatlılar</t>
         </is>
       </c>
       <c r="C194" s="11" t="inlineStr">
         <is>
-          <t>Tiramisu Dilim</t>
+          <t>Magnolia Çilek</t>
         </is>
       </c>
       <c r="D194" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E194" s="5" t="n"/>
       <c r="F194" s="5" t="n"/>
-      <c r="G194" s="9" t="n"/>
+      <c r="G194" s="9" t="inlineStr">
+        <is>
+          <t>Magnolia</t>
+        </is>
+      </c>
       <c r="H194" s="11" t="inlineStr">
         <is>
-          <t>Tiramisu Dilim</t>
+          <t>Magnolia Çilek</t>
         </is>
       </c>
     </row>
@@ -6482,11 +6482,11 @@
       </c>
       <c r="C195" s="11" t="inlineStr">
         <is>
-          <t>Magnolia Çilek</t>
+          <t>Magnolia Muzlu</t>
         </is>
       </c>
       <c r="D195" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E195" s="5" t="n"/>
       <c r="F195" s="5" t="n"/>
@@ -6497,7 +6497,7 @@
       </c>
       <c r="H195" s="11" t="inlineStr">
         <is>
-          <t>Magnolia Çilek</t>
+          <t>Magnolia Muzlu</t>
         </is>
       </c>
     </row>
@@ -6514,11 +6514,11 @@
       </c>
       <c r="C196" s="11" t="inlineStr">
         <is>
-          <t>Magnolia Muzlu</t>
+          <t>Magnolia Oreolu</t>
         </is>
       </c>
       <c r="D196" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E196" s="5" t="n"/>
       <c r="F196" s="5" t="n"/>
@@ -6529,7 +6529,7 @@
       </c>
       <c r="H196" s="11" t="inlineStr">
         <is>
-          <t>Magnolia Muzlu</t>
+          <t>Magnolia Oreolu</t>
         </is>
       </c>
     </row>
@@ -6546,11 +6546,11 @@
       </c>
       <c r="C197" s="11" t="inlineStr">
         <is>
-          <t>Magnolia Oreolu</t>
+          <t>Dubai Magnolia</t>
         </is>
       </c>
       <c r="D197" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E197" s="5" t="n"/>
       <c r="F197" s="5" t="n"/>
@@ -6561,7 +6561,7 @@
       </c>
       <c r="H197" s="11" t="inlineStr">
         <is>
-          <t>Magnolia Oreolu</t>
+          <t>Dubai Magnolia</t>
         </is>
       </c>
     </row>
@@ -6578,22 +6578,18 @@
       </c>
       <c r="C198" s="11" t="inlineStr">
         <is>
-          <t>Dubai Magnolia</t>
+          <t>Supangle</t>
         </is>
       </c>
       <c r="D198" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E198" s="5" t="n"/>
       <c r="F198" s="5" t="n"/>
-      <c r="G198" s="9" t="inlineStr">
-        <is>
-          <t>Magnolia</t>
-        </is>
-      </c>
+      <c r="G198" s="9" t="n"/>
       <c r="H198" s="11" t="inlineStr">
         <is>
-          <t>Dubai Magnolia</t>
+          <t>Supangle</t>
         </is>
       </c>
     </row>
@@ -6610,18 +6606,18 @@
       </c>
       <c r="C199" s="11" t="inlineStr">
         <is>
-          <t>Supangle</t>
+          <t>Profiterol Kase</t>
         </is>
       </c>
       <c r="D199" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E199" s="5" t="n"/>
       <c r="F199" s="5" t="n"/>
       <c r="G199" s="9" t="n"/>
       <c r="H199" s="11" t="inlineStr">
         <is>
-          <t>Supangle</t>
+          <t>Profiterol Kase</t>
         </is>
       </c>
     </row>
@@ -6638,18 +6634,18 @@
       </c>
       <c r="C200" s="11" t="inlineStr">
         <is>
-          <t>Profiterol Kase</t>
+          <t>Mozaik</t>
         </is>
       </c>
       <c r="D200" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E200" s="5" t="n"/>
       <c r="F200" s="5" t="n"/>
       <c r="G200" s="9" t="n"/>
       <c r="H200" s="11" t="inlineStr">
         <is>
-          <t>Profiterol Kase</t>
+          <t>Mozaik</t>
         </is>
       </c>
     </row>
@@ -6666,18 +6662,18 @@
       </c>
       <c r="C201" s="11" t="inlineStr">
         <is>
-          <t>Mozaik</t>
+          <t>Hasbahçe Tek</t>
         </is>
       </c>
       <c r="D201" s="4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E201" s="5" t="n"/>
       <c r="F201" s="5" t="n"/>
       <c r="G201" s="9" t="n"/>
       <c r="H201" s="11" t="inlineStr">
         <is>
-          <t>Mozaik</t>
+          <t>Hasbahçe Tek</t>
         </is>
       </c>
     </row>
@@ -6694,18 +6690,18 @@
       </c>
       <c r="C202" s="11" t="inlineStr">
         <is>
-          <t>Hasbahçe Tek</t>
+          <t>Fıstıklı Çikolatalı Tek</t>
         </is>
       </c>
       <c r="D202" s="4" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E202" s="5" t="n"/>
       <c r="F202" s="5" t="n"/>
       <c r="G202" s="9" t="n"/>
       <c r="H202" s="11" t="inlineStr">
         <is>
-          <t>Hasbahçe Tek</t>
+          <t>Fıstıklı Çikolatalı Tek</t>
         </is>
       </c>
     </row>
@@ -6722,18 +6718,18 @@
       </c>
       <c r="C203" s="11" t="inlineStr">
         <is>
-          <t>Fıstıklı Çikolatalı Tek</t>
+          <t>Kestaneli Tek</t>
         </is>
       </c>
       <c r="D203" s="4" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E203" s="5" t="n"/>
       <c r="F203" s="5" t="n"/>
       <c r="G203" s="9" t="n"/>
       <c r="H203" s="11" t="inlineStr">
         <is>
-          <t>Fıstıklı Çikolatalı Tek</t>
+          <t>Kestaneli Tek</t>
         </is>
       </c>
     </row>
@@ -6750,18 +6746,18 @@
       </c>
       <c r="C204" s="11" t="inlineStr">
         <is>
-          <t>Kestaneli Tek</t>
+          <t>Ganaj Tek</t>
         </is>
       </c>
       <c r="D204" s="4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E204" s="5" t="n"/>
       <c r="F204" s="5" t="n"/>
       <c r="G204" s="9" t="n"/>
       <c r="H204" s="11" t="inlineStr">
         <is>
-          <t>Kestaneli Tek</t>
+          <t>Ganaj Tek</t>
         </is>
       </c>
     </row>
@@ -6778,67 +6774,71 @@
       </c>
       <c r="C205" s="11" t="inlineStr">
         <is>
-          <t>Ganaj Tek</t>
+          <t>Latte (Porsiyon)</t>
         </is>
       </c>
       <c r="D205" s="4" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E205" s="5" t="n"/>
       <c r="F205" s="5" t="n"/>
       <c r="G205" s="9" t="n"/>
       <c r="H205" s="11" t="inlineStr">
         <is>
-          <t>Ganaj Tek</t>
+          <t xml:space="preserve">Latte </t>
         </is>
       </c>
     </row>
     <row r="206">
-      <c r="A206" s="11" t="inlineStr">
+      <c r="A206" s="8" t="inlineStr">
         <is>
           <t>Porsiyon Tatlılar</t>
         </is>
       </c>
-      <c r="B206" s="11" t="inlineStr">
-        <is>
-          <t>Porsiyon Tatlılar</t>
+      <c r="B206" s="8" t="inlineStr">
+        <is>
+          <t>Minik Tatlılar</t>
         </is>
       </c>
       <c r="C206" s="11" t="inlineStr">
         <is>
-          <t>Latte (Porsiyon)</t>
+          <t>Çikolatalı Ekler (Porsiyon)</t>
         </is>
       </c>
       <c r="D206" s="4" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="E206" s="5" t="n"/>
       <c r="F206" s="5" t="n"/>
-      <c r="G206" s="9" t="n"/>
+      <c r="G206" s="9" t="inlineStr">
+        <is>
+          <t>Ekler</t>
+        </is>
+      </c>
       <c r="H206" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Latte </t>
+          <t>Çikolatalı Ekler (kg)</t>
         </is>
       </c>
     </row>
     <row r="207">
-      <c r="A207" s="8" t="inlineStr">
+      <c r="A207" s="11" t="inlineStr">
         <is>
           <t>Porsiyon Tatlılar</t>
         </is>
       </c>
-      <c r="B207" s="8" t="inlineStr">
+      <c r="B207" s="11" t="inlineStr">
         <is>
           <t>Minik Tatlılar</t>
         </is>
       </c>
       <c r="C207" s="11" t="inlineStr">
         <is>
-          <t>Çikolatalı Ekler (Porsiyon)</t>
+          <t>Limonlu Ekler (Porsiyon)</t>
         </is>
       </c>
       <c r="D207" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E207" s="5" t="n"/>
       <c r="F207" s="5" t="n"/>
@@ -6849,7 +6849,7 @@
       </c>
       <c r="H207" s="11" t="inlineStr">
         <is>
-          <t>Çikolatalı Ekler (kg)</t>
+          <t>Limonlu Ekler (kg)</t>
         </is>
       </c>
     </row>
@@ -6866,11 +6866,11 @@
       </c>
       <c r="C208" s="11" t="inlineStr">
         <is>
-          <t>Limonlu Ekler (Porsiyon)</t>
+          <t>Beyaz Ekler</t>
         </is>
       </c>
       <c r="D208" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E208" s="5" t="n"/>
       <c r="F208" s="5" t="n"/>
@@ -6881,7 +6881,7 @@
       </c>
       <c r="H208" s="11" t="inlineStr">
         <is>
-          <t>Limonlu Ekler (kg)</t>
+          <t>Beyaz Ekler (kg)</t>
         </is>
       </c>
     </row>
@@ -6898,22 +6898,22 @@
       </c>
       <c r="C209" s="11" t="inlineStr">
         <is>
-          <t>Beyaz Ekler</t>
+          <t>Petifür</t>
         </is>
       </c>
       <c r="D209" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E209" s="5" t="n"/>
       <c r="F209" s="5" t="n"/>
       <c r="G209" s="9" t="inlineStr">
         <is>
-          <t>Ekler</t>
+          <t>Petifür &amp; Rulo</t>
         </is>
       </c>
       <c r="H209" s="11" t="inlineStr">
         <is>
-          <t>Beyaz Ekler (kg)</t>
+          <t>Petifür (kg)</t>
         </is>
       </c>
     </row>
@@ -6930,11 +6930,11 @@
       </c>
       <c r="C210" s="11" t="inlineStr">
         <is>
-          <t>Petifür</t>
+          <t>Rulo Petifür Muzlu</t>
         </is>
       </c>
       <c r="D210" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E210" s="5" t="n"/>
       <c r="F210" s="5" t="n"/>
@@ -6945,7 +6945,7 @@
       </c>
       <c r="H210" s="11" t="inlineStr">
         <is>
-          <t>Petifür (kg)</t>
+          <t>Rulo Petifür Muzlu (kg)</t>
         </is>
       </c>
     </row>
@@ -6962,11 +6962,11 @@
       </c>
       <c r="C211" s="11" t="inlineStr">
         <is>
-          <t>Rulo Petifür Muzlu</t>
+          <t>Rulo Petifür Çilek</t>
         </is>
       </c>
       <c r="D211" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E211" s="5" t="n"/>
       <c r="F211" s="5" t="n"/>
@@ -6977,7 +6977,7 @@
       </c>
       <c r="H211" s="11" t="inlineStr">
         <is>
-          <t>Rulo Petifür Muzlu (kg)</t>
+          <t>Rulo Petifür Çilek (kg)</t>
         </is>
       </c>
     </row>
@@ -6994,22 +6994,18 @@
       </c>
       <c r="C212" s="11" t="inlineStr">
         <is>
-          <t>Rulo Petifür Çilek</t>
+          <t>Çiko Limon Parfe</t>
         </is>
       </c>
       <c r="D212" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E212" s="5" t="n"/>
       <c r="F212" s="5" t="n"/>
-      <c r="G212" s="9" t="inlineStr">
-        <is>
-          <t>Petifür &amp; Rulo</t>
-        </is>
-      </c>
+      <c r="G212" s="9" t="n"/>
       <c r="H212" s="11" t="inlineStr">
         <is>
-          <t>Rulo Petifür Çilek (kg)</t>
+          <t>Çiko Limon Parfe (kg)</t>
         </is>
       </c>
     </row>
@@ -7026,18 +7022,22 @@
       </c>
       <c r="C213" s="11" t="inlineStr">
         <is>
-          <t>Çiko Limon Parfe</t>
+          <t>Çilekli Adet Rulo</t>
         </is>
       </c>
       <c r="D213" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E213" s="5" t="n"/>
       <c r="F213" s="5" t="n"/>
-      <c r="G213" s="9" t="n"/>
+      <c r="G213" s="9" t="inlineStr">
+        <is>
+          <t>Petifür &amp; Rulo</t>
+        </is>
+      </c>
       <c r="H213" s="11" t="inlineStr">
         <is>
-          <t>Çiko Limon Parfe (kg)</t>
+          <t>Çilekli Adet Rulo</t>
         </is>
       </c>
     </row>
@@ -7054,11 +7054,11 @@
       </c>
       <c r="C214" s="11" t="inlineStr">
         <is>
-          <t>Çilekli Adet Rulo</t>
+          <t>Muzlu Adet Rulo</t>
         </is>
       </c>
       <c r="D214" s="4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E214" s="5" t="n"/>
       <c r="F214" s="5" t="n"/>
@@ -7069,7 +7069,7 @@
       </c>
       <c r="H214" s="11" t="inlineStr">
         <is>
-          <t>Çilekli Adet Rulo</t>
+          <t>Muzlu Adet Rulo</t>
         </is>
       </c>
     </row>
@@ -7086,22 +7086,22 @@
       </c>
       <c r="C215" s="11" t="inlineStr">
         <is>
-          <t>Muzlu Adet Rulo</t>
+          <t>Krokanlı Şu Topu</t>
         </is>
       </c>
       <c r="D215" s="4" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E215" s="5" t="n"/>
       <c r="F215" s="5" t="n"/>
       <c r="G215" s="9" t="inlineStr">
         <is>
-          <t>Petifür &amp; Rulo</t>
+          <t>Şu Topu</t>
         </is>
       </c>
       <c r="H215" s="11" t="inlineStr">
         <is>
-          <t>Muzlu Adet Rulo</t>
+          <t>Krokanlı Şu Topu</t>
         </is>
       </c>
     </row>
@@ -7118,11 +7118,11 @@
       </c>
       <c r="C216" s="11" t="inlineStr">
         <is>
-          <t>Krokanlı Şu Topu</t>
+          <t>Çilekli Şu Topu</t>
         </is>
       </c>
       <c r="D216" s="4" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E216" s="5" t="n"/>
       <c r="F216" s="5" t="n"/>
@@ -7133,67 +7133,63 @@
       </c>
       <c r="H216" s="11" t="inlineStr">
         <is>
-          <t>Krokanlı Şu Topu</t>
+          <t>Çilekli Şu Topu</t>
         </is>
       </c>
     </row>
     <row r="217">
-      <c r="A217" s="11" t="inlineStr">
+      <c r="A217" s="2" t="inlineStr">
         <is>
           <t>Porsiyon Tatlılar</t>
         </is>
       </c>
-      <c r="B217" s="11" t="inlineStr">
-        <is>
-          <t>Minik Tatlılar</t>
+      <c r="B217" s="2" t="inlineStr">
+        <is>
+          <t>Sütlü Tatlı</t>
         </is>
       </c>
       <c r="C217" s="11" t="inlineStr">
         <is>
-          <t>Çilekli Şu Topu</t>
+          <t>Kazandibi</t>
         </is>
       </c>
       <c r="D217" s="4" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="E217" s="5" t="n"/>
       <c r="F217" s="5" t="n"/>
-      <c r="G217" s="9" t="inlineStr">
-        <is>
-          <t>Şu Topu</t>
-        </is>
-      </c>
+      <c r="G217" s="9" t="n"/>
       <c r="H217" s="11" t="inlineStr">
         <is>
-          <t>Çilekli Şu Topu</t>
+          <t>Kazandibi</t>
         </is>
       </c>
     </row>
     <row r="218">
-      <c r="A218" s="2" t="inlineStr">
+      <c r="A218" s="11" t="inlineStr">
         <is>
           <t>Porsiyon Tatlılar</t>
         </is>
       </c>
-      <c r="B218" s="2" t="inlineStr">
+      <c r="B218" s="11" t="inlineStr">
         <is>
           <t>Sütlü Tatlı</t>
         </is>
       </c>
       <c r="C218" s="11" t="inlineStr">
         <is>
-          <t>Kazandibi</t>
+          <t>Sütlaç</t>
         </is>
       </c>
       <c r="D218" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E218" s="5" t="n"/>
       <c r="F218" s="5" t="n"/>
       <c r="G218" s="9" t="n"/>
       <c r="H218" s="11" t="inlineStr">
         <is>
-          <t>Kazandibi</t>
+          <t>Sütlaç</t>
         </is>
       </c>
     </row>
@@ -7210,18 +7206,18 @@
       </c>
       <c r="C219" s="11" t="inlineStr">
         <is>
-          <t>Sütlaç</t>
+          <t>Aşure</t>
         </is>
       </c>
       <c r="D219" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E219" s="5" t="n"/>
       <c r="F219" s="5" t="n"/>
       <c r="G219" s="9" t="n"/>
       <c r="H219" s="11" t="inlineStr">
         <is>
-          <t>Sütlaç</t>
+          <t>Aşure</t>
         </is>
       </c>
     </row>
@@ -7233,23 +7229,27 @@
       </c>
       <c r="B220" s="11" t="inlineStr">
         <is>
-          <t>Sütlü Tatlı</t>
+          <t>Porsiyon Tatlılar</t>
         </is>
       </c>
       <c r="C220" s="11" t="inlineStr">
         <is>
-          <t>Aşure</t>
+          <t>Trileçe Frambuaz</t>
         </is>
       </c>
       <c r="D220" s="4" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E220" s="5" t="n"/>
       <c r="F220" s="5" t="n"/>
-      <c r="G220" s="9" t="n"/>
+      <c r="G220" s="9" t="inlineStr">
+        <is>
+          <t>Trileçe</t>
+        </is>
+      </c>
       <c r="H220" s="11" t="inlineStr">
         <is>
-          <t>Aşure</t>
+          <t xml:space="preserve"> Frambuaz Triliçe</t>
         </is>
       </c>
     </row>
@@ -7266,11 +7266,11 @@
       </c>
       <c r="C221" s="11" t="inlineStr">
         <is>
-          <t>Trileçe Frambuaz</t>
+          <t>Trileçe Karamel</t>
         </is>
       </c>
       <c r="D221" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E221" s="5" t="n"/>
       <c r="F221" s="5" t="n"/>
@@ -7280,38 +7280,6 @@
         </is>
       </c>
       <c r="H221" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Frambuaz Triliçe</t>
-        </is>
-      </c>
-    </row>
-    <row r="222">
-      <c r="A222" s="11" t="inlineStr">
-        <is>
-          <t>Porsiyon Tatlılar</t>
-        </is>
-      </c>
-      <c r="B222" s="11" t="inlineStr">
-        <is>
-          <t>Porsiyon Tatlılar</t>
-        </is>
-      </c>
-      <c r="C222" s="11" t="inlineStr">
-        <is>
-          <t>Trileçe Karamel</t>
-        </is>
-      </c>
-      <c r="D222" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="E222" s="5" t="n"/>
-      <c r="F222" s="5" t="n"/>
-      <c r="G222" s="9" t="inlineStr">
-        <is>
-          <t>Trileçe</t>
-        </is>
-      </c>
-      <c r="H222" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve"> Karamel Triliçe</t>
         </is>

</xml_diff>

<commit_message>
Faturada çıkan 5 ürünü kataloğa ekle
Eylül fatura mutabakatında Maslak'ın aldığı ama katalogda olmayan
kalemler: Machalı Şu Topu, Dome, Siyah Beyaz Çikolata Top, Panna Cotta
Shot Bardak, GR. Şu topu kuralıyla aynı: Beykent, Z.burnu ve S.beyli'de
gizli. Bölümlerin SIRA numaraları da baştan verildi.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/rapor-duzeni.xlsx
+++ b/rapor-duzeni.xlsx
@@ -500,7 +500,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H221"/>
+  <dimension ref="A1:H226"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -599,7 +599,9 @@
           <t>Karpatka</t>
         </is>
       </c>
-      <c r="D3" s="4" t="n"/>
+      <c r="D3" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="E3" s="5" t="n"/>
       <c r="F3" s="5" t="n"/>
       <c r="G3" s="9" t="n"/>
@@ -626,7 +628,7 @@
         </is>
       </c>
       <c r="D4" s="4" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="E4" s="5" t="n"/>
       <c r="F4" s="5" t="n"/>
@@ -654,7 +656,7 @@
         </is>
       </c>
       <c r="D5" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E5" s="5" t="n"/>
       <c r="F5" s="5" t="n"/>
@@ -682,7 +684,7 @@
         </is>
       </c>
       <c r="D6" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E6" s="5" t="n"/>
       <c r="F6" s="5" t="n"/>
@@ -710,7 +712,7 @@
         </is>
       </c>
       <c r="D7" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E7" s="5" t="n"/>
       <c r="F7" s="5" t="n"/>
@@ -738,7 +740,7 @@
         </is>
       </c>
       <c r="D8" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E8" s="5" t="n"/>
       <c r="F8" s="5" t="n"/>
@@ -766,7 +768,7 @@
         </is>
       </c>
       <c r="D9" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E9" s="5" t="n"/>
       <c r="F9" s="5" t="n"/>
@@ -794,7 +796,7 @@
         </is>
       </c>
       <c r="D10" s="4" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E10" s="5" t="n"/>
       <c r="F10" s="5" t="n"/>
@@ -822,7 +824,7 @@
         </is>
       </c>
       <c r="D11" s="4" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E11" s="5" t="n"/>
       <c r="F11" s="5" t="n"/>
@@ -850,7 +852,7 @@
         </is>
       </c>
       <c r="D12" s="4" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E12" s="5" t="n"/>
       <c r="F12" s="5" t="n"/>
@@ -878,7 +880,7 @@
         </is>
       </c>
       <c r="D13" s="4" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E13" s="5" t="n"/>
       <c r="F13" s="5" t="n"/>
@@ -906,7 +908,7 @@
         </is>
       </c>
       <c r="D14" s="4" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E14" s="5" t="n"/>
       <c r="F14" s="5" t="n"/>
@@ -934,7 +936,7 @@
         </is>
       </c>
       <c r="D15" s="4" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E15" s="5" t="n"/>
       <c r="F15" s="5" t="n"/>
@@ -962,7 +964,7 @@
         </is>
       </c>
       <c r="D16" s="4" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E16" s="5" t="n"/>
       <c r="F16" s="5" t="n"/>
@@ -990,7 +992,7 @@
         </is>
       </c>
       <c r="D17" s="4" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="E17" s="5" t="n"/>
       <c r="F17" s="5" t="n"/>
@@ -1018,7 +1020,7 @@
         </is>
       </c>
       <c r="D18" s="4" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E18" s="5" t="n"/>
       <c r="F18" s="5" t="n"/>
@@ -1046,7 +1048,7 @@
         </is>
       </c>
       <c r="D19" s="4" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E19" s="5" t="n"/>
       <c r="F19" s="5" t="n"/>
@@ -1074,7 +1076,7 @@
         </is>
       </c>
       <c r="D20" s="4" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E20" s="5" t="n"/>
       <c r="F20" s="5" t="n"/>
@@ -1102,7 +1104,7 @@
         </is>
       </c>
       <c r="D21" s="4" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E21" s="5" t="n"/>
       <c r="F21" s="5" t="n"/>
@@ -1130,7 +1132,7 @@
         </is>
       </c>
       <c r="D22" s="4" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E22" s="5" t="n"/>
       <c r="F22" s="5" t="n"/>
@@ -1158,7 +1160,7 @@
         </is>
       </c>
       <c r="D23" s="4" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E23" s="5" t="n"/>
       <c r="F23" s="5" t="n"/>
@@ -1186,7 +1188,7 @@
         </is>
       </c>
       <c r="D24" s="4" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E24" s="5" t="n"/>
       <c r="F24" s="5" t="n"/>
@@ -1214,7 +1216,7 @@
         </is>
       </c>
       <c r="D25" s="4" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="E25" s="5" t="n"/>
       <c r="F25" s="5" t="n"/>
@@ -1242,7 +1244,7 @@
         </is>
       </c>
       <c r="D26" s="4" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="E26" s="5" t="n"/>
       <c r="F26" s="5" t="n"/>
@@ -2650,7 +2652,7 @@
         </is>
       </c>
       <c r="D71" s="4" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="E71" s="5" t="n"/>
       <c r="F71" s="5" t="n"/>
@@ -2678,7 +2680,7 @@
         </is>
       </c>
       <c r="D72" s="4" t="n">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="E72" s="5" t="n"/>
       <c r="F72" s="5" t="n"/>
@@ -5710,7 +5712,7 @@
         </is>
       </c>
       <c r="D172" s="4" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E172" s="5" t="n"/>
       <c r="F172" s="5" t="n"/>
@@ -5742,7 +5744,7 @@
         </is>
       </c>
       <c r="D173" s="4" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E173" s="5" t="n"/>
       <c r="F173" s="5" t="n"/>
@@ -5774,7 +5776,7 @@
         </is>
       </c>
       <c r="D174" s="4" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="E174" s="5" t="n"/>
       <c r="F174" s="5" t="n"/>
@@ -5806,7 +5808,7 @@
         </is>
       </c>
       <c r="D175" s="4" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="E175" s="5" t="n"/>
       <c r="F175" s="5" t="n"/>
@@ -5834,7 +5836,7 @@
         </is>
       </c>
       <c r="D176" s="4" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E176" s="5" t="n"/>
       <c r="F176" s="5" t="n"/>
@@ -5862,7 +5864,7 @@
         </is>
       </c>
       <c r="D177" s="4" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E177" s="5" t="n"/>
       <c r="F177" s="5" t="n"/>
@@ -6790,162 +6792,134 @@
       </c>
     </row>
     <row r="206">
-      <c r="A206" s="8" t="inlineStr">
+      <c r="A206" t="inlineStr">
         <is>
           <t>Porsiyon Tatlılar</t>
         </is>
       </c>
-      <c r="B206" s="8" t="inlineStr">
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>Porsiyon Tatlılar</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>Dome</t>
+        </is>
+      </c>
+      <c r="D206" t="n">
+        <v>14</v>
+      </c>
+      <c r="H206" t="inlineStr">
+        <is>
+          <t>Dome</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>Porsiyon Tatlılar</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>Porsiyon Tatlılar</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>Siyah Beyaz Çikolata Top</t>
+        </is>
+      </c>
+      <c r="D207" t="n">
+        <v>15</v>
+      </c>
+      <c r="H207" t="inlineStr">
+        <is>
+          <t>Siyah Beyaz Çikolata Top</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>Porsiyon Tatlılar</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>Porsiyon Tatlılar</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>Panna Cotta Shot Bardak</t>
+        </is>
+      </c>
+      <c r="D208" t="n">
+        <v>16</v>
+      </c>
+      <c r="H208" t="inlineStr">
+        <is>
+          <t>Panna Cotta Shot Bardak</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>Porsiyon Tatlılar</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>Porsiyon Tatlılar</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>GR</t>
+        </is>
+      </c>
+      <c r="D209" t="n">
+        <v>17</v>
+      </c>
+      <c r="H209" t="inlineStr">
+        <is>
+          <t>GR</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="8" t="inlineStr">
+        <is>
+          <t>Porsiyon Tatlılar</t>
+        </is>
+      </c>
+      <c r="B210" s="8" t="inlineStr">
         <is>
           <t>Minik Tatlılar</t>
         </is>
       </c>
-      <c r="C206" s="11" t="inlineStr">
+      <c r="C210" s="11" t="inlineStr">
         <is>
           <t>Çikolatalı Ekler (Porsiyon)</t>
         </is>
       </c>
-      <c r="D206" s="4" t="n">
+      <c r="D210" s="4" t="n">
         <v>1</v>
-      </c>
-      <c r="E206" s="5" t="n"/>
-      <c r="F206" s="5" t="n"/>
-      <c r="G206" s="9" t="inlineStr">
-        <is>
-          <t>Ekler</t>
-        </is>
-      </c>
-      <c r="H206" s="11" t="inlineStr">
-        <is>
-          <t>Çikolatalı Ekler (kg)</t>
-        </is>
-      </c>
-    </row>
-    <row r="207">
-      <c r="A207" s="11" t="inlineStr">
-        <is>
-          <t>Porsiyon Tatlılar</t>
-        </is>
-      </c>
-      <c r="B207" s="11" t="inlineStr">
-        <is>
-          <t>Minik Tatlılar</t>
-        </is>
-      </c>
-      <c r="C207" s="11" t="inlineStr">
-        <is>
-          <t>Limonlu Ekler (Porsiyon)</t>
-        </is>
-      </c>
-      <c r="D207" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="E207" s="5" t="n"/>
-      <c r="F207" s="5" t="n"/>
-      <c r="G207" s="9" t="inlineStr">
-        <is>
-          <t>Ekler</t>
-        </is>
-      </c>
-      <c r="H207" s="11" t="inlineStr">
-        <is>
-          <t>Limonlu Ekler (kg)</t>
-        </is>
-      </c>
-    </row>
-    <row r="208">
-      <c r="A208" s="11" t="inlineStr">
-        <is>
-          <t>Porsiyon Tatlılar</t>
-        </is>
-      </c>
-      <c r="B208" s="11" t="inlineStr">
-        <is>
-          <t>Minik Tatlılar</t>
-        </is>
-      </c>
-      <c r="C208" s="11" t="inlineStr">
-        <is>
-          <t>Beyaz Ekler</t>
-        </is>
-      </c>
-      <c r="D208" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="E208" s="5" t="n"/>
-      <c r="F208" s="5" t="n"/>
-      <c r="G208" s="9" t="inlineStr">
-        <is>
-          <t>Ekler</t>
-        </is>
-      </c>
-      <c r="H208" s="11" t="inlineStr">
-        <is>
-          <t>Beyaz Ekler (kg)</t>
-        </is>
-      </c>
-    </row>
-    <row r="209">
-      <c r="A209" s="11" t="inlineStr">
-        <is>
-          <t>Porsiyon Tatlılar</t>
-        </is>
-      </c>
-      <c r="B209" s="11" t="inlineStr">
-        <is>
-          <t>Minik Tatlılar</t>
-        </is>
-      </c>
-      <c r="C209" s="11" t="inlineStr">
-        <is>
-          <t>Petifür</t>
-        </is>
-      </c>
-      <c r="D209" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="E209" s="5" t="n"/>
-      <c r="F209" s="5" t="n"/>
-      <c r="G209" s="9" t="inlineStr">
-        <is>
-          <t>Petifür &amp; Rulo</t>
-        </is>
-      </c>
-      <c r="H209" s="11" t="inlineStr">
-        <is>
-          <t>Petifür (kg)</t>
-        </is>
-      </c>
-    </row>
-    <row r="210">
-      <c r="A210" s="11" t="inlineStr">
-        <is>
-          <t>Porsiyon Tatlılar</t>
-        </is>
-      </c>
-      <c r="B210" s="11" t="inlineStr">
-        <is>
-          <t>Minik Tatlılar</t>
-        </is>
-      </c>
-      <c r="C210" s="11" t="inlineStr">
-        <is>
-          <t>Rulo Petifür Muzlu</t>
-        </is>
-      </c>
-      <c r="D210" s="4" t="n">
-        <v>5</v>
       </c>
       <c r="E210" s="5" t="n"/>
       <c r="F210" s="5" t="n"/>
       <c r="G210" s="9" t="inlineStr">
         <is>
-          <t>Petifür &amp; Rulo</t>
+          <t>Ekler</t>
         </is>
       </c>
       <c r="H210" s="11" t="inlineStr">
         <is>
-          <t>Rulo Petifür Muzlu (kg)</t>
+          <t>Çikolatalı Ekler (kg)</t>
         </is>
       </c>
     </row>
@@ -6962,22 +6936,22 @@
       </c>
       <c r="C211" s="11" t="inlineStr">
         <is>
-          <t>Rulo Petifür Çilek</t>
+          <t>Limonlu Ekler (Porsiyon)</t>
         </is>
       </c>
       <c r="D211" s="4" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E211" s="5" t="n"/>
       <c r="F211" s="5" t="n"/>
       <c r="G211" s="9" t="inlineStr">
         <is>
-          <t>Petifür &amp; Rulo</t>
+          <t>Ekler</t>
         </is>
       </c>
       <c r="H211" s="11" t="inlineStr">
         <is>
-          <t>Rulo Petifür Çilek (kg)</t>
+          <t>Limonlu Ekler (kg)</t>
         </is>
       </c>
     </row>
@@ -6994,18 +6968,22 @@
       </c>
       <c r="C212" s="11" t="inlineStr">
         <is>
-          <t>Çiko Limon Parfe</t>
+          <t>Beyaz Ekler</t>
         </is>
       </c>
       <c r="D212" s="4" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E212" s="5" t="n"/>
       <c r="F212" s="5" t="n"/>
-      <c r="G212" s="9" t="n"/>
+      <c r="G212" s="9" t="inlineStr">
+        <is>
+          <t>Ekler</t>
+        </is>
+      </c>
       <c r="H212" s="11" t="inlineStr">
         <is>
-          <t>Çiko Limon Parfe (kg)</t>
+          <t>Beyaz Ekler (kg)</t>
         </is>
       </c>
     </row>
@@ -7022,11 +7000,11 @@
       </c>
       <c r="C213" s="11" t="inlineStr">
         <is>
-          <t>Çilekli Adet Rulo</t>
+          <t>Petifür</t>
         </is>
       </c>
       <c r="D213" s="4" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="E213" s="5" t="n"/>
       <c r="F213" s="5" t="n"/>
@@ -7037,7 +7015,7 @@
       </c>
       <c r="H213" s="11" t="inlineStr">
         <is>
-          <t>Çilekli Adet Rulo</t>
+          <t>Petifür (kg)</t>
         </is>
       </c>
     </row>
@@ -7054,11 +7032,11 @@
       </c>
       <c r="C214" s="11" t="inlineStr">
         <is>
-          <t>Muzlu Adet Rulo</t>
+          <t>Rulo Petifür Muzlu</t>
         </is>
       </c>
       <c r="D214" s="4" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="E214" s="5" t="n"/>
       <c r="F214" s="5" t="n"/>
@@ -7069,7 +7047,7 @@
       </c>
       <c r="H214" s="11" t="inlineStr">
         <is>
-          <t>Muzlu Adet Rulo</t>
+          <t>Rulo Petifür Muzlu (kg)</t>
         </is>
       </c>
     </row>
@@ -7086,22 +7064,22 @@
       </c>
       <c r="C215" s="11" t="inlineStr">
         <is>
-          <t>Krokanlı Şu Topu</t>
+          <t>Rulo Petifür Çilek</t>
         </is>
       </c>
       <c r="D215" s="4" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E215" s="5" t="n"/>
       <c r="F215" s="5" t="n"/>
       <c r="G215" s="9" t="inlineStr">
         <is>
-          <t>Şu Topu</t>
+          <t>Petifür &amp; Rulo</t>
         </is>
       </c>
       <c r="H215" s="11" t="inlineStr">
         <is>
-          <t>Krokanlı Şu Topu</t>
+          <t>Rulo Petifür Çilek (kg)</t>
         </is>
       </c>
     </row>
@@ -7118,50 +7096,50 @@
       </c>
       <c r="C216" s="11" t="inlineStr">
         <is>
-          <t>Çilekli Şu Topu</t>
+          <t>Çiko Limon Parfe</t>
         </is>
       </c>
       <c r="D216" s="4" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="E216" s="5" t="n"/>
       <c r="F216" s="5" t="n"/>
-      <c r="G216" s="9" t="inlineStr">
-        <is>
-          <t>Şu Topu</t>
-        </is>
-      </c>
+      <c r="G216" s="9" t="n"/>
       <c r="H216" s="11" t="inlineStr">
         <is>
-          <t>Çilekli Şu Topu</t>
+          <t>Çiko Limon Parfe (kg)</t>
         </is>
       </c>
     </row>
     <row r="217">
-      <c r="A217" s="2" t="inlineStr">
+      <c r="A217" s="11" t="inlineStr">
         <is>
           <t>Porsiyon Tatlılar</t>
         </is>
       </c>
-      <c r="B217" s="2" t="inlineStr">
-        <is>
-          <t>Sütlü Tatlı</t>
+      <c r="B217" s="11" t="inlineStr">
+        <is>
+          <t>Minik Tatlılar</t>
         </is>
       </c>
       <c r="C217" s="11" t="inlineStr">
         <is>
-          <t>Kazandibi</t>
+          <t>Çilekli Adet Rulo</t>
         </is>
       </c>
       <c r="D217" s="4" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="E217" s="5" t="n"/>
       <c r="F217" s="5" t="n"/>
-      <c r="G217" s="9" t="n"/>
+      <c r="G217" s="9" t="inlineStr">
+        <is>
+          <t>Petifür &amp; Rulo</t>
+        </is>
+      </c>
       <c r="H217" s="11" t="inlineStr">
         <is>
-          <t>Kazandibi</t>
+          <t>Çilekli Adet Rulo</t>
         </is>
       </c>
     </row>
@@ -7173,23 +7151,27 @@
       </c>
       <c r="B218" s="11" t="inlineStr">
         <is>
-          <t>Sütlü Tatlı</t>
+          <t>Minik Tatlılar</t>
         </is>
       </c>
       <c r="C218" s="11" t="inlineStr">
         <is>
-          <t>Sütlaç</t>
+          <t>Muzlu Adet Rulo</t>
         </is>
       </c>
       <c r="D218" s="4" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="E218" s="5" t="n"/>
       <c r="F218" s="5" t="n"/>
-      <c r="G218" s="9" t="n"/>
+      <c r="G218" s="9" t="inlineStr">
+        <is>
+          <t>Petifür &amp; Rulo</t>
+        </is>
+      </c>
       <c r="H218" s="11" t="inlineStr">
         <is>
-          <t>Sütlaç</t>
+          <t>Muzlu Adet Rulo</t>
         </is>
       </c>
     </row>
@@ -7201,23 +7183,27 @@
       </c>
       <c r="B219" s="11" t="inlineStr">
         <is>
-          <t>Sütlü Tatlı</t>
+          <t>Minik Tatlılar</t>
         </is>
       </c>
       <c r="C219" s="11" t="inlineStr">
         <is>
-          <t>Aşure</t>
+          <t>Krokanlı Şu Topu</t>
         </is>
       </c>
       <c r="D219" s="4" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E219" s="5" t="n"/>
       <c r="F219" s="5" t="n"/>
-      <c r="G219" s="9" t="n"/>
+      <c r="G219" s="9" t="inlineStr">
+        <is>
+          <t>Şu Topu</t>
+        </is>
+      </c>
       <c r="H219" s="11" t="inlineStr">
         <is>
-          <t>Aşure</t>
+          <t>Krokanlı Şu Topu</t>
         </is>
       </c>
     </row>
@@ -7229,57 +7215,198 @@
       </c>
       <c r="B220" s="11" t="inlineStr">
         <is>
-          <t>Porsiyon Tatlılar</t>
+          <t>Minik Tatlılar</t>
         </is>
       </c>
       <c r="C220" s="11" t="inlineStr">
         <is>
-          <t>Trileçe Frambuaz</t>
+          <t>Çilekli Şu Topu</t>
         </is>
       </c>
       <c r="D220" s="4" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="E220" s="5" t="n"/>
       <c r="F220" s="5" t="n"/>
       <c r="G220" s="9" t="inlineStr">
         <is>
+          <t>Şu Topu</t>
+        </is>
+      </c>
+      <c r="H220" s="11" t="inlineStr">
+        <is>
+          <t>Çilekli Şu Topu</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>Porsiyon Tatlılar</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>Minik Tatlılar</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>Machalı Şu Topu</t>
+        </is>
+      </c>
+      <c r="D221" t="n">
+        <v>12</v>
+      </c>
+      <c r="H221" t="inlineStr">
+        <is>
+          <t>Machalı Şu Topu</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="2" t="inlineStr">
+        <is>
+          <t>Porsiyon Tatlılar</t>
+        </is>
+      </c>
+      <c r="B222" s="2" t="inlineStr">
+        <is>
+          <t>Sütlü Tatlı</t>
+        </is>
+      </c>
+      <c r="C222" s="11" t="inlineStr">
+        <is>
+          <t>Kazandibi</t>
+        </is>
+      </c>
+      <c r="D222" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E222" s="5" t="n"/>
+      <c r="F222" s="5" t="n"/>
+      <c r="G222" s="9" t="n"/>
+      <c r="H222" s="11" t="inlineStr">
+        <is>
+          <t>Kazandibi</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" s="11" t="inlineStr">
+        <is>
+          <t>Porsiyon Tatlılar</t>
+        </is>
+      </c>
+      <c r="B223" s="11" t="inlineStr">
+        <is>
+          <t>Sütlü Tatlı</t>
+        </is>
+      </c>
+      <c r="C223" s="11" t="inlineStr">
+        <is>
+          <t>Sütlaç</t>
+        </is>
+      </c>
+      <c r="D223" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E223" s="5" t="n"/>
+      <c r="F223" s="5" t="n"/>
+      <c r="G223" s="9" t="n"/>
+      <c r="H223" s="11" t="inlineStr">
+        <is>
+          <t>Sütlaç</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" s="11" t="inlineStr">
+        <is>
+          <t>Porsiyon Tatlılar</t>
+        </is>
+      </c>
+      <c r="B224" s="11" t="inlineStr">
+        <is>
+          <t>Sütlü Tatlı</t>
+        </is>
+      </c>
+      <c r="C224" s="11" t="inlineStr">
+        <is>
+          <t>Aşure</t>
+        </is>
+      </c>
+      <c r="D224" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="E224" s="5" t="n"/>
+      <c r="F224" s="5" t="n"/>
+      <c r="G224" s="9" t="n"/>
+      <c r="H224" s="11" t="inlineStr">
+        <is>
+          <t>Aşure</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" s="11" t="inlineStr">
+        <is>
+          <t>Porsiyon Tatlılar</t>
+        </is>
+      </c>
+      <c r="B225" s="11" t="inlineStr">
+        <is>
+          <t>Porsiyon Tatlılar</t>
+        </is>
+      </c>
+      <c r="C225" s="11" t="inlineStr">
+        <is>
+          <t>Trileçe Frambuaz</t>
+        </is>
+      </c>
+      <c r="D225" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="E225" s="5" t="n"/>
+      <c r="F225" s="5" t="n"/>
+      <c r="G225" s="9" t="inlineStr">
+        <is>
           <t>Trileçe</t>
         </is>
       </c>
-      <c r="H220" s="11" t="inlineStr">
+      <c r="H225" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve"> Frambuaz Triliçe</t>
         </is>
       </c>
     </row>
-    <row r="221">
-      <c r="A221" s="11" t="inlineStr">
+    <row r="226">
+      <c r="A226" s="11" t="inlineStr">
         <is>
           <t>Porsiyon Tatlılar</t>
         </is>
       </c>
-      <c r="B221" s="11" t="inlineStr">
+      <c r="B226" s="11" t="inlineStr">
         <is>
           <t>Porsiyon Tatlılar</t>
         </is>
       </c>
-      <c r="C221" s="11" t="inlineStr">
+      <c r="C226" s="11" t="inlineStr">
         <is>
           <t>Trileçe Karamel</t>
         </is>
       </c>
-      <c r="D221" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="E221" s="5" t="n"/>
-      <c r="F221" s="5" t="n"/>
-      <c r="G221" s="9" t="inlineStr">
+      <c r="D226" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="E226" s="5" t="n"/>
+      <c r="F226" s="5" t="n"/>
+      <c r="G226" s="9" t="inlineStr">
         <is>
           <t>Trileçe</t>
         </is>
       </c>
-      <c r="H221" s="11" t="inlineStr">
+      <c r="H226" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve"> Karamel Triliçe</t>
         </is>

</xml_diff>